<commit_message>
Update active PIV key checks for SP 800-78-5
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3124" uniqueCount="1309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1320" uniqueCount="1320">
   <si>
     <t>Document</t>
   </si>
@@ -3962,6 +3962,39 @@
   </si>
   <si>
     <t>No tags other than (0x01, 0x02, 0x04, 0x05, 0x06, 0x07, 0x08, 0xFE) are present</t>
+  </si>
+  <si>
+    <t>The PIV authentication key uses an allowed asymmetric algorithm under SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>78.1.current</t>
+  </si>
+  <si>
+    <t>The PIV authentication key size or curve is permitted by SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The digital signature key uses an allowed asymmetric algorithm under SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The digital signature key size or curve is permitted by SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The key management key uses an allowed asymmetric algorithm under SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The key management key size or curve is permitted by SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The asymmetric card authentication key uses an allowed algorithm under SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>The asymmetric card authentication key size or curve is permitted by SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>sp800_78_Test_1_current</t>
+  </si>
+  <si>
+    <t>Validate active PIV certificate public-key algorithms, sizes, curves, and RSA exponent against SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
   </si>
 </sst>
 </file>
@@ -4787,10 +4820,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:AMK490"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.8984375" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.69921875" style="2" customWidth="1"/>
@@ -4801,7 +4834,7 @@
     <col min="7" max="1025" width="8.5" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="5" customFormat="1" ns3:dyDescent="0.3">
       <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
@@ -4821,7 +4854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ns3:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>6</v>
       </c>
@@ -4835,7 +4868,7 @@
       <c r="E2" s="44"/>
       <c r="F2" s="44"/>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A3" s="45" t="s">
         <v>6</v>
       </c>
@@ -4849,7 +4882,7 @@
       <c r="E3" s="44"/>
       <c r="F3" s="44"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ns3:dyDescent="0.3">
       <c r="A4" s="45" t="s">
         <v>6</v>
       </c>
@@ -4863,7 +4896,7 @@
       <c r="E4" s="44"/>
       <c r="F4" s="44"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ns3:dyDescent="0.3">
       <c r="A5" s="45" t="s">
         <v>6</v>
       </c>
@@ -4881,7 +4914,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ns3:dyDescent="0.3">
       <c r="A6" s="45" t="s">
         <v>6</v>
       </c>
@@ -4899,7 +4932,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ns3:dyDescent="0.3">
       <c r="A7" s="45" t="s">
         <v>6</v>
       </c>
@@ -4917,7 +4950,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ns3:dyDescent="0.3">
       <c r="A8" s="45" t="s">
         <v>6</v>
       </c>
@@ -4935,7 +4968,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ns3:dyDescent="0.3">
       <c r="A9" s="45" t="s">
         <v>6</v>
       </c>
@@ -4953,7 +4986,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ns3:dyDescent="0.3">
       <c r="A10" s="45" t="s">
         <v>6</v>
       </c>
@@ -4971,7 +5004,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A11" s="45" t="s">
         <v>6</v>
       </c>
@@ -4989,7 +5022,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A12" s="45" t="s">
         <v>6</v>
       </c>
@@ -5007,7 +5040,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ns3:dyDescent="0.3">
       <c r="A13" s="45" t="s">
         <v>6</v>
       </c>
@@ -5025,7 +5058,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ns3:dyDescent="0.3">
       <c r="A14" s="45" t="s">
         <v>6</v>
       </c>
@@ -5043,7 +5076,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ns3:dyDescent="0.3">
       <c r="A15" s="45" t="s">
         <v>6</v>
       </c>
@@ -5061,7 +5094,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ns3:dyDescent="0.3">
       <c r="A16" s="45" t="s">
         <v>6</v>
       </c>
@@ -5075,7 +5108,7 @@
       <c r="E16" s="44"/>
       <c r="F16" s="44"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ns3:dyDescent="0.3">
       <c r="A17" s="45" t="s">
         <v>6</v>
       </c>
@@ -5089,7 +5122,7 @@
       <c r="E17" s="44"/>
       <c r="F17" s="44"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ns3:dyDescent="0.3">
       <c r="A18" s="45" t="s">
         <v>6</v>
       </c>
@@ -5107,7 +5140,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ns3:dyDescent="0.3">
       <c r="A19" s="45" t="s">
         <v>6</v>
       </c>
@@ -5125,7 +5158,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ns3:dyDescent="0.3">
       <c r="A20" s="45" t="s">
         <v>6</v>
       </c>
@@ -5143,7 +5176,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ns3:dyDescent="0.3">
       <c r="A21" s="45" t="s">
         <v>6</v>
       </c>
@@ -5161,7 +5194,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ns3:dyDescent="0.3">
       <c r="A22" s="45" t="s">
         <v>6</v>
       </c>
@@ -5179,7 +5212,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ns3:dyDescent="0.3">
       <c r="A23" s="45" t="s">
         <v>6</v>
       </c>
@@ -5197,7 +5230,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ns3:dyDescent="0.3">
       <c r="A24" s="54" t="s">
         <v>6</v>
       </c>
@@ -5215,7 +5248,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ns3:dyDescent="0.3">
       <c r="A25" s="45" t="s">
         <v>6</v>
       </c>
@@ -5233,7 +5266,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ns3:dyDescent="0.3">
       <c r="A26" s="54" t="s">
         <v>6</v>
       </c>
@@ -5251,7 +5284,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ns3:dyDescent="0.3">
       <c r="A27" s="54" t="s">
         <v>6</v>
       </c>
@@ -5269,7 +5302,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ns3:dyDescent="0.3">
       <c r="A28" s="54" t="s">
         <v>6</v>
       </c>
@@ -5287,7 +5320,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ns3:dyDescent="0.3">
       <c r="A29" s="54" t="s">
         <v>6</v>
       </c>
@@ -5305,7 +5338,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ns3:dyDescent="0.3">
       <c r="A30" s="45" t="s">
         <v>6</v>
       </c>
@@ -5323,7 +5356,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ns3:dyDescent="0.3">
       <c r="A31" s="45" t="s">
         <v>6</v>
       </c>
@@ -5341,7 +5374,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ns3:dyDescent="0.3">
       <c r="A32" s="54" t="s">
         <v>6</v>
       </c>
@@ -5359,7 +5392,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ns3:dyDescent="0.3">
       <c r="A33" s="54" t="s">
         <v>6</v>
       </c>
@@ -5377,7 +5410,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ns3:dyDescent="0.3">
       <c r="A34" s="54" t="s">
         <v>6</v>
       </c>
@@ -5395,7 +5428,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" ns3:dyDescent="0.3">
       <c r="A35" s="54" t="s">
         <v>6</v>
       </c>
@@ -5413,7 +5446,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ns3:dyDescent="0.3">
       <c r="A36" s="45" t="s">
         <v>6</v>
       </c>
@@ -5431,7 +5464,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ns3:dyDescent="0.3">
       <c r="A37" s="45" t="s">
         <v>6</v>
       </c>
@@ -5449,7 +5482,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A38" s="45" t="s">
         <v>6</v>
       </c>
@@ -5467,7 +5500,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ns3:dyDescent="0.3">
       <c r="A39" s="45" t="s">
         <v>6</v>
       </c>
@@ -5485,7 +5518,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ns3:dyDescent="0.3">
       <c r="A40" s="45" t="s">
         <v>6</v>
       </c>
@@ -5503,7 +5536,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A41" s="45" t="s">
         <v>6</v>
       </c>
@@ -5521,7 +5554,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" ns3:dyDescent="0.3">
       <c r="A42" s="45" t="s">
         <v>6</v>
       </c>
@@ -5539,7 +5572,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" ns3:dyDescent="0.3">
       <c r="A43" s="45" t="s">
         <v>117</v>
       </c>
@@ -5557,7 +5590,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" ns3:dyDescent="0.3">
       <c r="A44" s="45" t="s">
         <v>6</v>
       </c>
@@ -5571,7 +5604,7 @@
       <c r="E44" s="44"/>
       <c r="F44" s="44"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" ns3:dyDescent="0.3">
       <c r="A45" s="45" t="s">
         <v>6</v>
       </c>
@@ -5585,7 +5618,7 @@
       <c r="E45" s="44"/>
       <c r="F45" s="44"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" ns3:dyDescent="0.3">
       <c r="A46" s="45" t="s">
         <v>6</v>
       </c>
@@ -5603,7 +5636,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" ns3:dyDescent="0.3">
       <c r="A47" s="45" t="s">
         <v>6</v>
       </c>
@@ -5621,7 +5654,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" ns3:dyDescent="0.3">
       <c r="A48" s="45" t="s">
         <v>6</v>
       </c>
@@ -5639,7 +5672,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" ns3:dyDescent="0.3">
       <c r="A49" s="45" t="s">
         <v>6</v>
       </c>
@@ -5657,7 +5690,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A50" s="45" t="s">
         <v>6</v>
       </c>
@@ -5675,7 +5708,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" ns3:dyDescent="0.3">
       <c r="A51" s="45" t="s">
         <v>6</v>
       </c>
@@ -5693,7 +5726,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" ns3:dyDescent="0.3">
       <c r="A52" s="45" t="s">
         <v>6</v>
       </c>
@@ -5711,7 +5744,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" ns3:dyDescent="0.3">
       <c r="A53" s="45" t="s">
         <v>6</v>
       </c>
@@ -5729,7 +5762,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" ns3:dyDescent="0.3">
       <c r="A54" s="45" t="s">
         <v>6</v>
       </c>
@@ -5747,7 +5780,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" ns3:dyDescent="0.3">
       <c r="A55" s="45" t="s">
         <v>117</v>
       </c>
@@ -5765,7 +5798,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" ns3:dyDescent="0.3">
       <c r="A56" s="45" t="s">
         <v>6</v>
       </c>
@@ -5779,7 +5812,7 @@
       <c r="E56" s="44"/>
       <c r="F56" s="44"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" ns3:dyDescent="0.3">
       <c r="A57" s="45" t="s">
         <v>6</v>
       </c>
@@ -5793,7 +5826,7 @@
       <c r="E57" s="44"/>
       <c r="F57" s="44"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" ns3:dyDescent="0.3">
       <c r="A58" s="45" t="s">
         <v>6</v>
       </c>
@@ -5811,7 +5844,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" ns3:dyDescent="0.3">
       <c r="A59" s="45" t="s">
         <v>6</v>
       </c>
@@ -5829,7 +5862,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" ns3:dyDescent="0.3">
       <c r="A60" s="45" t="s">
         <v>6</v>
       </c>
@@ -5847,7 +5880,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" ns3:dyDescent="0.3">
       <c r="A61" s="45" t="s">
         <v>6</v>
       </c>
@@ -5865,7 +5898,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" ns3:dyDescent="0.3">
       <c r="A62" s="45" t="s">
         <v>6</v>
       </c>
@@ -5883,7 +5916,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" ns3:dyDescent="0.3">
       <c r="A63" s="45" t="s">
         <v>6</v>
       </c>
@@ -5901,7 +5934,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" ns3:dyDescent="0.3">
       <c r="A64" s="45" t="s">
         <v>6</v>
       </c>
@@ -5915,7 +5948,7 @@
       <c r="E64" s="44"/>
       <c r="F64" s="44"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" ns3:dyDescent="0.3">
       <c r="A65" s="45" t="s">
         <v>6</v>
       </c>
@@ -5929,7 +5962,7 @@
       <c r="E65" s="44"/>
       <c r="F65" s="44"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" ns3:dyDescent="0.3">
       <c r="A66" s="45" t="s">
         <v>6</v>
       </c>
@@ -5947,7 +5980,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" ns3:dyDescent="0.3">
       <c r="A67" s="45" t="s">
         <v>6</v>
       </c>
@@ -5965,7 +5998,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" ns3:dyDescent="0.3">
       <c r="A68" s="45" t="s">
         <v>6</v>
       </c>
@@ -5983,7 +6016,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" ns3:dyDescent="0.3">
       <c r="A69" s="45" t="s">
         <v>6</v>
       </c>
@@ -6001,7 +6034,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" ns3:dyDescent="0.3">
       <c r="A70" s="45" t="s">
         <v>6</v>
       </c>
@@ -6019,7 +6052,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" ns3:dyDescent="0.3">
       <c r="A71" s="45" t="s">
         <v>6</v>
       </c>
@@ -6037,7 +6070,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" ns3:dyDescent="0.3">
       <c r="A72" s="54" t="s">
         <v>6</v>
       </c>
@@ -6055,7 +6088,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" ns3:dyDescent="0.3">
       <c r="A73" s="54" t="s">
         <v>6</v>
       </c>
@@ -6073,7 +6106,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" ns3:dyDescent="0.3">
       <c r="A74" s="45" t="s">
         <v>6</v>
       </c>
@@ -6091,7 +6124,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" ns3:dyDescent="0.3">
       <c r="A75" s="45" t="s">
         <v>6</v>
       </c>
@@ -6109,7 +6142,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" ns3:dyDescent="0.3">
       <c r="A76" s="45" t="s">
         <v>6</v>
       </c>
@@ -6127,7 +6160,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" ns3:dyDescent="0.3">
       <c r="A77" s="45" t="s">
         <v>117</v>
       </c>
@@ -6145,7 +6178,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" ns3:dyDescent="0.3">
       <c r="A78" s="45" t="s">
         <v>6</v>
       </c>
@@ -6159,7 +6192,7 @@
       <c r="E78" s="44"/>
       <c r="F78" s="44"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" ns3:dyDescent="0.3">
       <c r="A79" s="45" t="s">
         <v>6</v>
       </c>
@@ -6173,7 +6206,7 @@
       <c r="E79" s="44"/>
       <c r="F79" s="44"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" ns3:dyDescent="0.3">
       <c r="A80" s="45" t="s">
         <v>6</v>
       </c>
@@ -6191,7 +6224,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" ns3:dyDescent="0.3">
       <c r="A81" s="45" t="s">
         <v>6</v>
       </c>
@@ -6209,7 +6242,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" ns3:dyDescent="0.3">
       <c r="A82" s="45" t="s">
         <v>6</v>
       </c>
@@ -6227,7 +6260,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" ns3:dyDescent="0.3">
       <c r="A83" s="45" t="s">
         <v>6</v>
       </c>
@@ -6245,7 +6278,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" ns3:dyDescent="0.3">
       <c r="A84" s="45" t="s">
         <v>6</v>
       </c>
@@ -6263,7 +6296,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" ns3:dyDescent="0.3">
       <c r="A85" s="45" t="s">
         <v>6</v>
       </c>
@@ -6281,7 +6314,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" ns3:dyDescent="0.3">
       <c r="A86" s="45" t="s">
         <v>6</v>
       </c>
@@ -6299,7 +6332,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" ns3:dyDescent="0.3">
       <c r="A87" s="45" t="s">
         <v>117</v>
       </c>
@@ -6317,7 +6350,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" ns3:dyDescent="0.3">
       <c r="A88" s="45" t="s">
         <v>6</v>
       </c>
@@ -6331,7 +6364,7 @@
       <c r="E88" s="44"/>
       <c r="F88" s="44"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" ns3:dyDescent="0.3">
       <c r="A89" s="45" t="s">
         <v>6</v>
       </c>
@@ -6345,7 +6378,7 @@
       <c r="E89" s="44"/>
       <c r="F89" s="44"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" ns3:dyDescent="0.3">
       <c r="A90" s="45" t="s">
         <v>6</v>
       </c>
@@ -6363,7 +6396,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" ns3:dyDescent="0.3">
       <c r="A91" s="45" t="s">
         <v>6</v>
       </c>
@@ -6381,7 +6414,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" ns3:dyDescent="0.3">
       <c r="A92" s="45" t="s">
         <v>6</v>
       </c>
@@ -6399,7 +6432,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" ns3:dyDescent="0.3">
       <c r="A93" s="45" t="s">
         <v>6</v>
       </c>
@@ -6417,7 +6450,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A94" s="45" t="s">
         <v>6</v>
       </c>
@@ -6435,7 +6468,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" ns3:dyDescent="0.3">
       <c r="A95" s="45" t="s">
         <v>6</v>
       </c>
@@ -6453,7 +6486,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" ns3:dyDescent="0.3">
       <c r="A96" s="45" t="s">
         <v>6</v>
       </c>
@@ -6471,7 +6504,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" ns3:dyDescent="0.3">
       <c r="A97" s="45" t="s">
         <v>6</v>
       </c>
@@ -6489,7 +6522,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" ns3:dyDescent="0.3">
       <c r="A98" s="45" t="s">
         <v>6</v>
       </c>
@@ -6507,7 +6540,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" ns3:dyDescent="0.3">
       <c r="A99" s="45" t="s">
         <v>117</v>
       </c>
@@ -6525,7 +6558,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" ns3:dyDescent="0.3">
       <c r="A100" s="45" t="s">
         <v>6</v>
       </c>
@@ -6539,7 +6572,7 @@
       <c r="E100" s="44"/>
       <c r="F100" s="44"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" ns3:dyDescent="0.3">
       <c r="A101" s="45" t="s">
         <v>6</v>
       </c>
@@ -6553,7 +6586,7 @@
       <c r="E101" s="44"/>
       <c r="F101" s="44"/>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" ns3:dyDescent="0.3">
       <c r="A102" s="45" t="s">
         <v>6</v>
       </c>
@@ -6571,7 +6604,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" ns3:dyDescent="0.3">
       <c r="A103" s="45" t="s">
         <v>6</v>
       </c>
@@ -6589,7 +6622,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" ns3:dyDescent="0.3">
       <c r="A104" s="45" t="s">
         <v>6</v>
       </c>
@@ -6607,7 +6640,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" ns3:dyDescent="0.3">
       <c r="A105" s="45" t="s">
         <v>6</v>
       </c>
@@ -6625,7 +6658,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A106" s="45" t="s">
         <v>6</v>
       </c>
@@ -6643,7 +6676,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" ns3:dyDescent="0.3">
       <c r="A107" s="45" t="s">
         <v>6</v>
       </c>
@@ -6661,7 +6694,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" ns3:dyDescent="0.3">
       <c r="A108" s="45" t="s">
         <v>6</v>
       </c>
@@ -6679,7 +6712,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" ns3:dyDescent="0.3">
       <c r="A109" s="45" t="s">
         <v>6</v>
       </c>
@@ -6697,7 +6730,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" ns3:dyDescent="0.3">
       <c r="A110" s="45" t="s">
         <v>6</v>
       </c>
@@ -6715,7 +6748,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" ns3:dyDescent="0.3">
       <c r="A111" s="45" t="s">
         <v>117</v>
       </c>
@@ -6733,7 +6766,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" ns3:dyDescent="0.3">
       <c r="A112" s="45" t="s">
         <v>6</v>
       </c>
@@ -6747,7 +6780,7 @@
       <c r="E112" s="44"/>
       <c r="F112" s="44"/>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" ns3:dyDescent="0.3">
       <c r="A113" s="45" t="s">
         <v>6</v>
       </c>
@@ -6761,7 +6794,7 @@
       <c r="E113" s="44"/>
       <c r="F113" s="44"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" ns3:dyDescent="0.3">
       <c r="A114" s="45" t="s">
         <v>6</v>
       </c>
@@ -6779,7 +6812,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" ns3:dyDescent="0.3">
       <c r="A115" s="45" t="s">
         <v>6</v>
       </c>
@@ -6797,7 +6830,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" ns3:dyDescent="0.3">
       <c r="A116" s="45" t="s">
         <v>6</v>
       </c>
@@ -6815,7 +6848,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" ns3:dyDescent="0.3">
       <c r="A117" s="45" t="s">
         <v>6</v>
       </c>
@@ -6833,7 +6866,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A118" s="45" t="s">
         <v>6</v>
       </c>
@@ -6851,7 +6884,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" ns3:dyDescent="0.3">
       <c r="A119" s="45" t="s">
         <v>6</v>
       </c>
@@ -6869,7 +6902,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" ns3:dyDescent="0.3">
       <c r="A120" s="45" t="s">
         <v>6</v>
       </c>
@@ -6887,7 +6920,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" ns3:dyDescent="0.3">
       <c r="A121" s="45" t="s">
         <v>6</v>
       </c>
@@ -6905,7 +6938,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" ns3:dyDescent="0.3">
       <c r="A122" s="45" t="s">
         <v>6</v>
       </c>
@@ -6923,7 +6956,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" ns3:dyDescent="0.3">
       <c r="A123" s="45" t="s">
         <v>117</v>
       </c>
@@ -6941,7 +6974,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" ns3:dyDescent="0.3">
       <c r="A124" s="45" t="s">
         <v>6</v>
       </c>
@@ -6955,7 +6988,7 @@
       <c r="E124" s="44"/>
       <c r="F124" s="44"/>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" ns3:dyDescent="0.3">
       <c r="A125" s="45" t="s">
         <v>6</v>
       </c>
@@ -6969,7 +7002,7 @@
       <c r="E125" s="44"/>
       <c r="F125" s="44"/>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" ns3:dyDescent="0.3">
       <c r="A126" s="45" t="s">
         <v>6</v>
       </c>
@@ -6987,7 +7020,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" ns3:dyDescent="0.3">
       <c r="A127" s="45" t="s">
         <v>6</v>
       </c>
@@ -7005,7 +7038,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" ns3:dyDescent="0.3">
       <c r="A128" s="45" t="s">
         <v>6</v>
       </c>
@@ -7023,7 +7056,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" ns3:dyDescent="0.3">
       <c r="A129" s="45" t="s">
         <v>6</v>
       </c>
@@ -7041,7 +7074,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" ns3:dyDescent="0.3">
       <c r="A130" s="45" t="s">
         <v>6</v>
       </c>
@@ -7059,7 +7092,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" ns3:dyDescent="0.3">
       <c r="A131" s="45" t="s">
         <v>6</v>
       </c>
@@ -7077,7 +7110,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" ns3:dyDescent="0.3">
       <c r="A132" s="54" t="s">
         <v>6</v>
       </c>
@@ -7095,7 +7128,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" ns3:dyDescent="0.3">
       <c r="A133" s="45" t="s">
         <v>6</v>
       </c>
@@ -7113,7 +7146,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A134" s="45" t="s">
         <v>6</v>
       </c>
@@ -7131,7 +7164,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" ns3:dyDescent="0.3">
       <c r="A135" s="45" t="s">
         <v>6</v>
       </c>
@@ -7145,7 +7178,7 @@
       <c r="E135" s="44"/>
       <c r="F135" s="44"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" ns3:dyDescent="0.3">
       <c r="A136" s="45" t="s">
         <v>6</v>
       </c>
@@ -7159,7 +7192,7 @@
       <c r="E136" s="44"/>
       <c r="F136" s="44"/>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" ns3:dyDescent="0.3">
       <c r="A137" s="45" t="s">
         <v>6</v>
       </c>
@@ -7177,7 +7210,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" ns3:dyDescent="0.3">
       <c r="A138" s="45" t="s">
         <v>6</v>
       </c>
@@ -7195,7 +7228,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" ns3:dyDescent="0.3">
       <c r="A139" s="45" t="s">
         <v>6</v>
       </c>
@@ -7213,7 +7246,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" ns3:dyDescent="0.3">
       <c r="A140" s="45" t="s">
         <v>6</v>
       </c>
@@ -7231,7 +7264,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" ns3:dyDescent="0.3">
       <c r="A141" s="45" t="s">
         <v>6</v>
       </c>
@@ -7249,7 +7282,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" ns3:dyDescent="0.3">
       <c r="A142" s="45" t="s">
         <v>6</v>
       </c>
@@ -7267,7 +7300,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" ns3:dyDescent="0.3">
       <c r="A143" s="54" t="s">
         <v>6</v>
       </c>
@@ -7285,7 +7318,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" ns3:dyDescent="0.3">
       <c r="A144" s="45" t="s">
         <v>6</v>
       </c>
@@ -7303,7 +7336,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A145" s="45" t="s">
         <v>6</v>
       </c>
@@ -7321,7 +7354,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" ns3:dyDescent="0.3">
       <c r="A146" s="45" t="s">
         <v>117</v>
       </c>
@@ -7339,7 +7372,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" ns3:dyDescent="0.3">
       <c r="A147" s="45" t="s">
         <v>117</v>
       </c>
@@ -7353,7 +7386,7 @@
       <c r="E147" s="46"/>
       <c r="F147" s="44"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" ns3:dyDescent="0.3">
       <c r="A148" s="45" t="s">
         <v>6</v>
       </c>
@@ -7367,7 +7400,7 @@
       <c r="E148" s="46"/>
       <c r="F148" s="44"/>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" ns3:dyDescent="0.3">
       <c r="A149" s="45" t="s">
         <v>6</v>
       </c>
@@ -7385,7 +7418,7 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="150" spans="1:6" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" ht="16.2" customHeight="1" ns3:dyDescent="0.3">
       <c r="A150" s="45" t="s">
         <v>6</v>
       </c>
@@ -7403,7 +7436,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" ns3:dyDescent="0.3">
       <c r="A151" s="45" t="s">
         <v>6</v>
       </c>
@@ -7421,7 +7454,7 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" ns3:dyDescent="0.3">
       <c r="A152" s="45" t="s">
         <v>6</v>
       </c>
@@ -7435,7 +7468,7 @@
       <c r="E152" s="46"/>
       <c r="F152" s="46"/>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" ns3:dyDescent="0.3">
       <c r="A153" s="45" t="s">
         <v>6</v>
       </c>
@@ -7449,7 +7482,7 @@
       <c r="E153" s="46"/>
       <c r="F153" s="46"/>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" ns3:dyDescent="0.3">
       <c r="A154" s="45" t="s">
         <v>6</v>
       </c>
@@ -7463,7 +7496,7 @@
       <c r="E154" s="46"/>
       <c r="F154" s="46"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" ns3:dyDescent="0.3">
       <c r="A155" s="42" t="s">
         <v>6</v>
       </c>
@@ -7477,7 +7510,7 @@
       <c r="E155" s="48"/>
       <c r="F155" s="46"/>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" ns3:dyDescent="0.3">
       <c r="A156" s="49" t="s">
         <v>6</v>
       </c>
@@ -7491,7 +7524,7 @@
       <c r="E156" s="46"/>
       <c r="F156" s="46"/>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" ns3:dyDescent="0.3">
       <c r="A157" s="45" t="s">
         <v>6</v>
       </c>
@@ -7505,7 +7538,7 @@
       <c r="E157" s="46"/>
       <c r="F157" s="46"/>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" ns3:dyDescent="0.3">
       <c r="A158" s="45" t="s">
         <v>6</v>
       </c>
@@ -7523,7 +7556,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" ns3:dyDescent="0.3">
       <c r="A159" s="45" t="s">
         <v>6</v>
       </c>
@@ -7541,7 +7574,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" ns3:dyDescent="0.3">
       <c r="A160" s="45" t="s">
         <v>6</v>
       </c>
@@ -7559,7 +7592,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" ns3:dyDescent="0.3">
       <c r="A161" s="45" t="s">
         <v>6</v>
       </c>
@@ -7577,7 +7610,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" ns3:dyDescent="0.3">
       <c r="A162" s="45" t="s">
         <v>6</v>
       </c>
@@ -7595,7 +7628,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" ns3:dyDescent="0.3">
       <c r="A163" s="45" t="s">
         <v>6</v>
       </c>
@@ -7609,7 +7642,7 @@
       <c r="E163" s="46"/>
       <c r="F163" s="46"/>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" ns3:dyDescent="0.3">
       <c r="A164" s="45" t="s">
         <v>6</v>
       </c>
@@ -7627,7 +7660,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" ns3:dyDescent="0.3">
       <c r="A165" s="45" t="s">
         <v>6</v>
       </c>
@@ -7645,7 +7678,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="166" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A166" s="45" t="s">
         <v>6</v>
       </c>
@@ -7663,7 +7696,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" ns3:dyDescent="0.3">
       <c r="A167" s="45" t="s">
         <v>6</v>
       </c>
@@ -7681,7 +7714,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="168" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A168" s="45" t="s">
         <v>6</v>
       </c>
@@ -7699,7 +7732,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" ns3:dyDescent="0.3">
       <c r="A169" s="45" t="s">
         <v>6</v>
       </c>
@@ -7717,7 +7750,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" ns3:dyDescent="0.3">
       <c r="A170" s="45" t="s">
         <v>6</v>
       </c>
@@ -7735,7 +7768,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="171" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A171" s="45" t="s">
         <v>6</v>
       </c>
@@ -7753,7 +7786,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" ns3:dyDescent="0.3">
       <c r="A172" s="45" t="s">
         <v>6</v>
       </c>
@@ -7771,7 +7804,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A173" s="45" t="s">
         <v>6</v>
       </c>
@@ -7789,7 +7822,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="174" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A174" s="45" t="s">
         <v>6</v>
       </c>
@@ -7807,7 +7840,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" ns3:dyDescent="0.3">
       <c r="A175" s="45" t="s">
         <v>6</v>
       </c>
@@ -7825,7 +7858,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" ns3:dyDescent="0.3">
       <c r="A176" s="45" t="s">
         <v>6</v>
       </c>
@@ -7839,7 +7872,7 @@
       <c r="E176" s="46"/>
       <c r="F176" s="46"/>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" ns3:dyDescent="0.3">
       <c r="A177" s="45" t="s">
         <v>6</v>
       </c>
@@ -7853,7 +7886,7 @@
       <c r="E177" s="46"/>
       <c r="F177" s="46"/>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" ns3:dyDescent="0.3">
       <c r="A178" s="45" t="s">
         <v>6</v>
       </c>
@@ -7871,7 +7904,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" ns3:dyDescent="0.3">
       <c r="A179" s="45" t="s">
         <v>6</v>
       </c>
@@ -7889,7 +7922,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" ns3:dyDescent="0.3">
       <c r="A180" s="45" t="s">
         <v>6</v>
       </c>
@@ -7907,7 +7940,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" ns3:dyDescent="0.3">
       <c r="A181" s="45" t="s">
         <v>6</v>
       </c>
@@ -7925,7 +7958,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" ns3:dyDescent="0.3">
       <c r="A182" s="45" t="s">
         <v>6</v>
       </c>
@@ -7939,7 +7972,7 @@
       <c r="E182" s="46"/>
       <c r="F182" s="46"/>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" ns3:dyDescent="0.3">
       <c r="A183" s="45" t="s">
         <v>6</v>
       </c>
@@ -7957,7 +7990,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" ns3:dyDescent="0.3">
       <c r="A184" s="45" t="s">
         <v>6</v>
       </c>
@@ -7975,7 +8008,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A185" s="45" t="s">
         <v>6</v>
       </c>
@@ -7993,7 +8026,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" ns3:dyDescent="0.3">
       <c r="A186" s="45" t="s">
         <v>6</v>
       </c>
@@ -8011,7 +8044,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A187" s="45" t="s">
         <v>6</v>
       </c>
@@ -8029,7 +8062,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" ns3:dyDescent="0.3">
       <c r="A188" s="45" t="s">
         <v>6</v>
       </c>
@@ -8047,7 +8080,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" ns3:dyDescent="0.3">
       <c r="A189" s="45" t="s">
         <v>6</v>
       </c>
@@ -8065,7 +8098,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A190" s="45" t="s">
         <v>6</v>
       </c>
@@ -8083,7 +8116,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" ns3:dyDescent="0.3">
       <c r="A191" s="45" t="s">
         <v>6</v>
       </c>
@@ -8101,7 +8134,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A192" s="45" t="s">
         <v>6</v>
       </c>
@@ -8119,7 +8152,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A193" s="45" t="s">
         <v>6</v>
       </c>
@@ -8137,7 +8170,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:6" ns3:dyDescent="0.3">
       <c r="A194" s="45" t="s">
         <v>6</v>
       </c>
@@ -8155,7 +8188,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:6" ns3:dyDescent="0.3">
       <c r="A195" s="45" t="s">
         <v>6</v>
       </c>
@@ -8169,7 +8202,7 @@
       <c r="E195" s="46"/>
       <c r="F195" s="46"/>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:6" ns3:dyDescent="0.3">
       <c r="A196" s="45" t="s">
         <v>6</v>
       </c>
@@ -8183,7 +8216,7 @@
       <c r="E196" s="46"/>
       <c r="F196" s="46"/>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:6" ns3:dyDescent="0.3">
       <c r="A197" s="45" t="s">
         <v>6</v>
       </c>
@@ -8201,7 +8234,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:6" ns3:dyDescent="0.3">
       <c r="A198" s="45" t="s">
         <v>6</v>
       </c>
@@ -8219,7 +8252,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:6" ns3:dyDescent="0.3">
       <c r="A199" s="45" t="s">
         <v>6</v>
       </c>
@@ -8237,7 +8270,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:6" ns3:dyDescent="0.3">
       <c r="A200" s="45" t="s">
         <v>6</v>
       </c>
@@ -8255,7 +8288,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:6" ns3:dyDescent="0.3">
       <c r="A201" s="45" t="s">
         <v>6</v>
       </c>
@@ -8269,7 +8302,7 @@
       <c r="E201" s="46"/>
       <c r="F201" s="46"/>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:6" ns3:dyDescent="0.3">
       <c r="A202" s="45" t="s">
         <v>6</v>
       </c>
@@ -8287,7 +8320,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:6" ns3:dyDescent="0.3">
       <c r="A203" s="45" t="s">
         <v>6</v>
       </c>
@@ -8305,7 +8338,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:6" ns3:dyDescent="0.3">
       <c r="A204" s="45" t="s">
         <v>6</v>
       </c>
@@ -8323,7 +8356,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:6" ns3:dyDescent="0.3">
       <c r="A205" s="45" t="s">
         <v>6</v>
       </c>
@@ -8341,7 +8374,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="206" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A206" s="45" t="s">
         <v>6</v>
       </c>
@@ -8359,7 +8392,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:6" ns3:dyDescent="0.3">
       <c r="A207" s="45" t="s">
         <v>6</v>
       </c>
@@ -8377,7 +8410,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" ns3:dyDescent="0.3">
       <c r="A208" s="45" t="s">
         <v>6</v>
       </c>
@@ -8395,7 +8428,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="209" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A209" s="45" t="s">
         <v>6</v>
       </c>
@@ -8413,7 +8446,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" ns3:dyDescent="0.3">
       <c r="A210" s="45" t="s">
         <v>6</v>
       </c>
@@ -8431,7 +8464,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="211" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A211" s="45" t="s">
         <v>6</v>
       </c>
@@ -8449,7 +8482,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="212" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A212" s="45" t="s">
         <v>6</v>
       </c>
@@ -8467,7 +8500,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" ns3:dyDescent="0.3">
       <c r="A213" s="45" t="s">
         <v>6</v>
       </c>
@@ -8485,7 +8518,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="214" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A214" s="45" t="s">
         <v>6</v>
       </c>
@@ -8499,7 +8532,7 @@
       <c r="E214" s="46"/>
       <c r="F214" s="46"/>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" ns3:dyDescent="0.3">
       <c r="A215" s="45" t="s">
         <v>6</v>
       </c>
@@ -8513,7 +8546,7 @@
       <c r="E215" s="46"/>
       <c r="F215" s="46"/>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" ns3:dyDescent="0.3">
       <c r="A216" s="45" t="s">
         <v>6</v>
       </c>
@@ -8531,7 +8564,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" ns3:dyDescent="0.3">
       <c r="A217" s="45" t="s">
         <v>6</v>
       </c>
@@ -8549,7 +8582,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" ns3:dyDescent="0.3">
       <c r="A218" s="45" t="s">
         <v>6</v>
       </c>
@@ -8567,7 +8600,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="219" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A219" s="45" t="s">
         <v>6</v>
       </c>
@@ -8585,7 +8618,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="220" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A220" s="45" t="s">
         <v>6</v>
       </c>
@@ -8603,7 +8636,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:6" ns3:dyDescent="0.3">
       <c r="A221" s="45" t="s">
         <v>6</v>
       </c>
@@ -8621,7 +8654,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:6" ns3:dyDescent="0.3">
       <c r="A222" s="45" t="s">
         <v>6</v>
       </c>
@@ -8639,7 +8672,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:6" ns3:dyDescent="0.3">
       <c r="A223" s="45" t="s">
         <v>6</v>
       </c>
@@ -8657,7 +8690,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="224" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A224" s="45" t="s">
         <v>6</v>
       </c>
@@ -8675,7 +8708,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:6" ns3:dyDescent="0.3">
       <c r="A225" s="45" t="s">
         <v>6</v>
       </c>
@@ -8693,7 +8726,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:6" ns3:dyDescent="0.3">
       <c r="A226" s="45" t="s">
         <v>6</v>
       </c>
@@ -8711,7 +8744,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:6" ns3:dyDescent="0.3">
       <c r="A227" s="45" t="s">
         <v>6</v>
       </c>
@@ -8729,7 +8762,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:6" ns3:dyDescent="0.3">
       <c r="A228" s="45" t="s">
         <v>6</v>
       </c>
@@ -8743,7 +8776,7 @@
       <c r="E228" s="46"/>
       <c r="F228" s="46"/>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:6" ns3:dyDescent="0.3">
       <c r="A229" s="45" t="s">
         <v>6</v>
       </c>
@@ -8761,7 +8794,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:6" ns3:dyDescent="0.3">
       <c r="A230" s="45" t="s">
         <v>6</v>
       </c>
@@ -8779,7 +8812,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:6" ns3:dyDescent="0.3">
       <c r="A231" s="45" t="s">
         <v>6</v>
       </c>
@@ -8797,7 +8830,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:6" ns3:dyDescent="0.3">
       <c r="A232" s="45" t="s">
         <v>6</v>
       </c>
@@ -8815,7 +8848,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:6" ns3:dyDescent="0.3">
       <c r="A233" s="45" t="s">
         <v>6</v>
       </c>
@@ -8833,7 +8866,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:6" ns3:dyDescent="0.3">
       <c r="A234" s="45" t="s">
         <v>6</v>
       </c>
@@ -8851,7 +8884,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:6" ns3:dyDescent="0.3">
       <c r="A235" s="45" t="s">
         <v>6</v>
       </c>
@@ -8869,7 +8902,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:6" ns3:dyDescent="0.3">
       <c r="A236" s="45" t="s">
         <v>6</v>
       </c>
@@ -8887,7 +8920,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:6" ns3:dyDescent="0.3">
       <c r="A237" s="45" t="s">
         <v>6</v>
       </c>
@@ -8905,7 +8938,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:6" ns3:dyDescent="0.3">
       <c r="A238" s="45" t="s">
         <v>6</v>
       </c>
@@ -8923,7 +8956,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:6" ns3:dyDescent="0.3">
       <c r="A239" s="45" t="s">
         <v>6</v>
       </c>
@@ -8941,7 +8974,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:6" ns3:dyDescent="0.3">
       <c r="A240" s="45" t="s">
         <v>6</v>
       </c>
@@ -8955,7 +8988,7 @@
       <c r="E240" s="46"/>
       <c r="F240" s="46"/>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:6" ns3:dyDescent="0.3">
       <c r="A241" s="45" t="s">
         <v>6</v>
       </c>
@@ -8973,7 +9006,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:6" ns3:dyDescent="0.3">
       <c r="A242" s="45" t="s">
         <v>6</v>
       </c>
@@ -8991,7 +9024,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="243" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A243" s="45" t="s">
         <v>6</v>
       </c>
@@ -9005,7 +9038,7 @@
       <c r="E243" s="46"/>
       <c r="F243" s="46"/>
     </row>
-    <row r="244" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A244" s="45" t="s">
         <v>6</v>
       </c>
@@ -9021,7 +9054,7 @@
       <c r="E244" s="45"/>
       <c r="F244" s="45"/>
     </row>
-    <row r="245" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A245" s="45" t="s">
         <v>6</v>
       </c>
@@ -9035,7 +9068,7 @@
       <c r="E245" s="46"/>
       <c r="F245" s="46"/>
     </row>
-    <row r="246" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A246" s="45" t="s">
         <v>6</v>
       </c>
@@ -9049,7 +9082,7 @@
       <c r="E246" s="46"/>
       <c r="F246" s="46"/>
     </row>
-    <row r="247" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A247" s="45" t="s">
         <v>6</v>
       </c>
@@ -9067,7 +9100,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="248" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A248" s="45" t="s">
         <v>6</v>
       </c>
@@ -9085,7 +9118,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="249" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A249" s="45" t="s">
         <v>6</v>
       </c>
@@ -9103,7 +9136,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="250" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A250" s="45" t="s">
         <v>6</v>
       </c>
@@ -9121,7 +9154,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="251" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A251" s="45" t="s">
         <v>6</v>
       </c>
@@ -9135,7 +9168,7 @@
       <c r="E251" s="46"/>
       <c r="F251" s="46"/>
     </row>
-    <row r="252" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A252" s="45" t="s">
         <v>6</v>
       </c>
@@ -9153,7 +9186,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="253" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A253" s="45" t="s">
         <v>6</v>
       </c>
@@ -9171,7 +9204,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="254" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A254" s="45" t="s">
         <v>6</v>
       </c>
@@ -9189,7 +9222,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="255" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A255" s="45" t="s">
         <v>6</v>
       </c>
@@ -9207,7 +9240,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="256" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A256" s="45" t="s">
         <v>6</v>
       </c>
@@ -9221,7 +9254,7 @@
       <c r="E256" s="46"/>
       <c r="F256" s="46"/>
     </row>
-    <row r="257" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A257" s="45" t="s">
         <v>6</v>
       </c>
@@ -9239,7 +9272,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="258" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A258" s="45" t="s">
         <v>6</v>
       </c>
@@ -9257,7 +9290,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:6" ns3:dyDescent="0.3">
       <c r="A259" s="53" t="s">
         <v>6</v>
       </c>
@@ -9271,7 +9304,7 @@
       <c r="E259" s="48"/>
       <c r="F259" s="46"/>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:6" ns3:dyDescent="0.3">
       <c r="A260" s="45" t="s">
         <v>6</v>
       </c>
@@ -9285,7 +9318,7 @@
       <c r="E260" s="46"/>
       <c r="F260" s="46"/>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:6" ns3:dyDescent="0.3">
       <c r="A261" s="45" t="s">
         <v>6</v>
       </c>
@@ -9299,7 +9332,7 @@
       <c r="E261" s="46"/>
       <c r="F261" s="46"/>
     </row>
-    <row r="262" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A262" s="45" t="s">
         <v>6</v>
       </c>
@@ -9317,7 +9350,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:6" ns3:dyDescent="0.3">
       <c r="A263" s="45" t="s">
         <v>6</v>
       </c>
@@ -9335,7 +9368,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:6" ns3:dyDescent="0.3">
       <c r="A264" s="45" t="s">
         <v>6</v>
       </c>
@@ -9353,7 +9386,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="265" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A265" s="45" t="s">
         <v>6</v>
       </c>
@@ -9371,7 +9404,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:6" ns3:dyDescent="0.3">
       <c r="A266" s="45" t="s">
         <v>6</v>
       </c>
@@ -9389,7 +9422,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:6" ns3:dyDescent="0.3">
       <c r="A267" s="45" t="s">
         <v>6</v>
       </c>
@@ -9407,7 +9440,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="268" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A268" s="45" t="s">
         <v>6</v>
       </c>
@@ -9425,7 +9458,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="269" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:6" s="7" customFormat="1" ns3:dyDescent="0.3">
       <c r="A269" s="45" t="s">
         <v>6</v>
       </c>
@@ -9439,7 +9472,7 @@
       <c r="E269" s="46"/>
       <c r="F269" s="46"/>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:6" ns3:dyDescent="0.3">
       <c r="A270" s="45" t="s">
         <v>6</v>
       </c>
@@ -9457,7 +9490,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="271" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A271" s="45" t="s">
         <v>6</v>
       </c>
@@ -9475,7 +9508,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="272" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A272" s="45" t="s">
         <v>6</v>
       </c>
@@ -9493,7 +9526,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="273" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A273" s="45" t="s">
         <v>6</v>
       </c>
@@ -9511,7 +9544,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="274" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A274" s="45" t="s">
         <v>6</v>
       </c>
@@ -9529,7 +9562,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:6" ns3:dyDescent="0.3">
       <c r="A275" s="45" t="s">
         <v>6</v>
       </c>
@@ -9547,7 +9580,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:6" ns3:dyDescent="0.3">
       <c r="A276" s="45" t="s">
         <v>6</v>
       </c>
@@ -9561,7 +9594,7 @@
       <c r="E276" s="46"/>
       <c r="F276" s="46"/>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:6" ns3:dyDescent="0.3">
       <c r="A277" s="45" t="s">
         <v>6</v>
       </c>
@@ -9575,7 +9608,7 @@
       <c r="E277" s="46"/>
       <c r="F277" s="46"/>
     </row>
-    <row r="278" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A278" s="45" t="s">
         <v>6</v>
       </c>
@@ -9593,7 +9626,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:6" ns3:dyDescent="0.3">
       <c r="A279" s="45" t="s">
         <v>6</v>
       </c>
@@ -9611,7 +9644,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:6" ns3:dyDescent="0.3">
       <c r="A280" s="45" t="s">
         <v>6</v>
       </c>
@@ -9629,7 +9662,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="281" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A281" s="45" t="s">
         <v>6</v>
       </c>
@@ -9647,7 +9680,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:6" ns3:dyDescent="0.3">
       <c r="A282" s="45" t="s">
         <v>6</v>
       </c>
@@ -9665,7 +9698,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:6" ns3:dyDescent="0.3">
       <c r="A283" s="45" t="s">
         <v>6</v>
       </c>
@@ -9683,7 +9716,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:6" ns3:dyDescent="0.3">
       <c r="A284" s="45" t="s">
         <v>6</v>
       </c>
@@ -9701,7 +9734,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="285" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A285" s="45" t="s">
         <v>6</v>
       </c>
@@ -9719,7 +9752,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="286" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:6" s="7" customFormat="1" ns3:dyDescent="0.3">
       <c r="A286" s="45" t="s">
         <v>6</v>
       </c>
@@ -9733,7 +9766,7 @@
       <c r="E286" s="46"/>
       <c r="F286" s="46"/>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:6" ns3:dyDescent="0.3">
       <c r="A287" s="45" t="s">
         <v>6</v>
       </c>
@@ -9751,7 +9784,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="288" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A288" s="45" t="s">
         <v>6</v>
       </c>
@@ -9769,7 +9802,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="289" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A289" s="45" t="s">
         <v>6</v>
       </c>
@@ -9787,7 +9820,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="290" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A290" s="45" t="s">
         <v>6</v>
       </c>
@@ -9805,7 +9838,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="291" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A291" s="45" t="s">
         <v>6</v>
       </c>
@@ -9823,7 +9856,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="292" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A292" s="45" t="s">
         <v>6</v>
       </c>
@@ -9841,7 +9874,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:6" ns3:dyDescent="0.3">
       <c r="A293" s="45" t="s">
         <v>6</v>
       </c>
@@ -9859,7 +9892,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:6" ns3:dyDescent="0.3">
       <c r="A294" s="45" t="s">
         <v>6</v>
       </c>
@@ -9877,7 +9910,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:6" ns3:dyDescent="0.3">
       <c r="A295" s="45" t="s">
         <v>6</v>
       </c>
@@ -9895,7 +9928,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:6" ns3:dyDescent="0.3">
       <c r="A296" s="45" t="s">
         <v>6</v>
       </c>
@@ -9909,7 +9942,7 @@
       <c r="E296" s="46"/>
       <c r="F296" s="46"/>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:6" ns3:dyDescent="0.3">
       <c r="A297" s="45" t="s">
         <v>6</v>
       </c>
@@ -9923,7 +9956,7 @@
       <c r="E297" s="46"/>
       <c r="F297" s="46"/>
     </row>
-    <row r="298" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A298" s="45" t="s">
         <v>6</v>
       </c>
@@ -9941,7 +9974,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:6" ns3:dyDescent="0.3">
       <c r="A299" s="45" t="s">
         <v>6</v>
       </c>
@@ -9959,7 +9992,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:6" ns3:dyDescent="0.3">
       <c r="A300" s="45" t="s">
         <v>6</v>
       </c>
@@ -9977,7 +10010,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="301" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A301" s="45" t="s">
         <v>6</v>
       </c>
@@ -9995,7 +10028,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:6" ns3:dyDescent="0.3">
       <c r="A302" s="45" t="s">
         <v>6</v>
       </c>
@@ -10013,7 +10046,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:6" ns3:dyDescent="0.3">
       <c r="A303" s="45" t="s">
         <v>6</v>
       </c>
@@ -10031,7 +10064,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:6" ns3:dyDescent="0.3">
       <c r="A304" s="45" t="s">
         <v>6</v>
       </c>
@@ -10049,7 +10082,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="305" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A305" s="45" t="s">
         <v>6</v>
       </c>
@@ -10067,7 +10100,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="306" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:6" s="7" customFormat="1" ns3:dyDescent="0.3">
       <c r="A306" s="45" t="s">
         <v>6</v>
       </c>
@@ -10081,7 +10114,7 @@
       <c r="E306" s="46"/>
       <c r="F306" s="46"/>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:6" ns3:dyDescent="0.3">
       <c r="A307" s="45" t="s">
         <v>6</v>
       </c>
@@ -10099,7 +10132,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="308" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A308" s="45" t="s">
         <v>6</v>
       </c>
@@ -10117,7 +10150,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="309" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A309" s="45" t="s">
         <v>6</v>
       </c>
@@ -10135,7 +10168,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="310" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A310" s="45" t="s">
         <v>6</v>
       </c>
@@ -10153,7 +10186,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="311" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A311" s="45" t="s">
         <v>6</v>
       </c>
@@ -10171,7 +10204,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="312" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A312" s="45" t="s">
         <v>6</v>
       </c>
@@ -10189,7 +10222,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="313" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A313" s="45" t="s">
         <v>6</v>
       </c>
@@ -10207,7 +10240,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:6" ns3:dyDescent="0.3">
       <c r="A314" s="45" t="s">
         <v>6</v>
       </c>
@@ -10225,7 +10258,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:6" ns3:dyDescent="0.3">
       <c r="A315" s="45" t="s">
         <v>6</v>
       </c>
@@ -10243,7 +10276,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:6" ns3:dyDescent="0.3">
       <c r="A316" s="45" t="s">
         <v>6</v>
       </c>
@@ -10257,7 +10290,7 @@
       <c r="E316" s="46"/>
       <c r="F316" s="46"/>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:6" ns3:dyDescent="0.3">
       <c r="A317" s="45" t="s">
         <v>6</v>
       </c>
@@ -10271,7 +10304,7 @@
       <c r="E317" s="46"/>
       <c r="F317" s="46"/>
     </row>
-    <row r="318" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A318" s="45" t="s">
         <v>6</v>
       </c>
@@ -10289,7 +10322,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:6" ns3:dyDescent="0.3">
       <c r="A319" s="45" t="s">
         <v>6</v>
       </c>
@@ -10303,7 +10336,7 @@
       <c r="E319" s="46"/>
       <c r="F319" s="46"/>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:6" ns3:dyDescent="0.3">
       <c r="A320" s="45" t="s">
         <v>6</v>
       </c>
@@ -10321,7 +10354,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="321" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A321" s="45" t="s">
         <v>6</v>
       </c>
@@ -10339,7 +10372,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="322" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A322" s="45" t="s">
         <v>6</v>
       </c>
@@ -10357,7 +10390,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="323" spans="1:1025" ht="30" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:1025" ht="30" ns3:dyDescent="0.3">
       <c r="A323" s="45" t="s">
         <v>6</v>
       </c>
@@ -10375,7 +10408,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="324" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A324" s="45" t="s">
         <v>6</v>
       </c>
@@ -10393,7 +10426,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="325" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A325" s="45" t="s">
         <v>6</v>
       </c>
@@ -10411,7 +10444,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="326" spans="1:1025" ht="45" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:1025" ht="45" ns3:dyDescent="0.3">
       <c r="A326" s="45" t="s">
         <v>6</v>
       </c>
@@ -10429,7 +10462,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="327" spans="1:1025" s="40" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:1025" s="40" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A327" s="45" t="s">
         <v>6</v>
       </c>
@@ -11466,7 +11499,7 @@
       <c r="AMJ327" s="39"/>
       <c r="AMK327" s="39"/>
     </row>
-    <row r="328" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A328" s="45" t="s">
         <v>6</v>
       </c>
@@ -11480,7 +11513,7 @@
       <c r="E328" s="46"/>
       <c r="F328" s="46"/>
     </row>
-    <row r="329" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A329" s="45" t="s">
         <v>6</v>
       </c>
@@ -11494,7 +11527,7 @@
       <c r="E329" s="46"/>
       <c r="F329" s="46"/>
     </row>
-    <row r="330" spans="1:1025" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:1025" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A330" s="45" t="s">
         <v>6</v>
       </c>
@@ -11512,7 +11545,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="331" spans="1:1025" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:1025" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A331" s="45" t="s">
         <v>6</v>
       </c>
@@ -11530,7 +11563,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="332" spans="1:1025" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:1025" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A332" s="45" t="s">
         <v>6</v>
       </c>
@@ -11548,7 +11581,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="333" spans="1:1025" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:1025" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A333" s="45" t="s">
         <v>6</v>
       </c>
@@ -11566,7 +11599,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="334" spans="1:1025" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:1025" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A334" s="45" t="s">
         <v>6</v>
       </c>
@@ -11584,7 +11617,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="335" spans="1:1025" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:1025" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A335" s="45" t="s">
         <v>6</v>
       </c>
@@ -11602,7 +11635,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="336" spans="1:1025" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:1025" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A336" s="45" t="s">
         <v>6</v>
       </c>
@@ -11620,7 +11653,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="337" spans="1:6" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:6" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A337" s="45" t="s">
         <v>6</v>
       </c>
@@ -11638,7 +11671,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="338" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:6" s="7" customFormat="1" ns3:dyDescent="0.3">
       <c r="A338" s="45" t="s">
         <v>6</v>
       </c>
@@ -11652,7 +11685,7 @@
       <c r="E338" s="46"/>
       <c r="F338" s="46"/>
     </row>
-    <row r="339" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A339" s="45" t="s">
         <v>6</v>
       </c>
@@ -11670,7 +11703,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="340" spans="1:6" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:6" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A340" s="45" t="s">
         <v>6</v>
       </c>
@@ -11688,7 +11721,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="341" spans="1:6" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:6" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A341" s="45" t="s">
         <v>6</v>
       </c>
@@ -11706,7 +11739,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="342" spans="1:6" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:6" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A342" s="45" t="s">
         <v>6</v>
       </c>
@@ -11724,7 +11757,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="343" spans="1:6" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:6" s="6" customFormat="1" ht="45" ns3:dyDescent="0.3">
       <c r="A343" s="45" t="s">
         <v>6</v>
       </c>
@@ -11742,7 +11775,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="344" spans="1:6" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:6" s="6" customFormat="1" ht="45" ns3:dyDescent="0.3">
       <c r="A344" s="45" t="s">
         <v>6</v>
       </c>
@@ -11760,7 +11793,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="345" spans="1:6" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:6" s="6" customFormat="1" ht="30" ns3:dyDescent="0.3">
       <c r="A345" s="45" t="s">
         <v>6</v>
       </c>
@@ -11778,7 +11811,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="346" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:6" s="6" customFormat="1" ns3:dyDescent="0.3">
       <c r="A346" s="45" t="s">
         <v>6</v>
       </c>
@@ -11796,7 +11829,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="347" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:6" ns3:dyDescent="0.3">
       <c r="A347" s="45" t="s">
         <v>6</v>
       </c>
@@ -11814,7 +11847,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="348" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:6" ht="31.2" ns3:dyDescent="0.3">
       <c r="A348" s="53" t="s">
         <v>6</v>
       </c>
@@ -11828,7 +11861,7 @@
       <c r="E348" s="46"/>
       <c r="F348" s="46"/>
     </row>
-    <row r="349" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:6" ns3:dyDescent="0.3">
       <c r="A349" s="45" t="s">
         <v>6</v>
       </c>
@@ -11842,7 +11875,7 @@
       <c r="E349" s="46"/>
       <c r="F349" s="46"/>
     </row>
-    <row r="350" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:6" ns3:dyDescent="0.3">
       <c r="A350" s="45" t="s">
         <v>6</v>
       </c>
@@ -11856,7 +11889,7 @@
       <c r="E350" s="46"/>
       <c r="F350" s="46"/>
     </row>
-    <row r="351" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:6" ht="60" ns3:dyDescent="0.3">
       <c r="A351" s="45" t="s">
         <v>6</v>
       </c>
@@ -11874,7 +11907,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="352" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:6" ns3:dyDescent="0.3">
       <c r="A352" s="45" t="s">
         <v>6</v>
       </c>
@@ -11882,17 +11915,17 @@
         <v>671</v>
       </c>
       <c r="C352" s="52" t="s">
-        <v>672</v>
-      </c>
-      <c r="D352" s="45">
-        <v>78.099999999999994</v>
+        <v>1309</v>
+      </c>
+      <c r="D352" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E352" s="45"/>
       <c r="F352" s="45" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="353" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:6" ns3:dyDescent="0.3">
       <c r="A353" s="45" t="s">
         <v>6</v>
       </c>
@@ -11900,17 +11933,17 @@
         <v>673</v>
       </c>
       <c r="C353" s="52" t="s">
-        <v>674</v>
-      </c>
-      <c r="D353" s="45">
-        <v>78.099999999999994</v>
+        <v>1311</v>
+      </c>
+      <c r="D353" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E353" s="45"/>
       <c r="F353" s="45" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="354" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:6" ns3:dyDescent="0.3">
       <c r="A354" s="45" t="s">
         <v>6</v>
       </c>
@@ -11924,7 +11957,7 @@
       <c r="E354" s="46"/>
       <c r="F354" s="46"/>
     </row>
-    <row r="355" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:6" ns3:dyDescent="0.3">
       <c r="A355" s="45" t="s">
         <v>6</v>
       </c>
@@ -11938,7 +11971,7 @@
       <c r="E355" s="46"/>
       <c r="F355" s="46"/>
     </row>
-    <row r="356" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:6" ns3:dyDescent="0.3">
       <c r="A356" s="45" t="s">
         <v>6</v>
       </c>
@@ -11956,7 +11989,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="357" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:6" ns3:dyDescent="0.3">
       <c r="A357" s="45" t="s">
         <v>6</v>
       </c>
@@ -11974,7 +12007,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="358" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:6" ns3:dyDescent="0.3">
       <c r="A358" s="45" t="s">
         <v>6</v>
       </c>
@@ -11992,7 +12025,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="359" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:6" ns3:dyDescent="0.3">
       <c r="A359" s="45" t="s">
         <v>6</v>
       </c>
@@ -12010,7 +12043,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="360" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:6" ns3:dyDescent="0.3">
       <c r="A360" s="45" t="s">
         <v>6</v>
       </c>
@@ -12028,7 +12061,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="361" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:6" ns3:dyDescent="0.3">
       <c r="A361" s="45" t="s">
         <v>6</v>
       </c>
@@ -12042,7 +12075,7 @@
       <c r="E361" s="46"/>
       <c r="F361" s="46"/>
     </row>
-    <row r="362" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:6" ns3:dyDescent="0.3">
       <c r="A362" s="45" t="s">
         <v>6</v>
       </c>
@@ -12060,7 +12093,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="363" spans="1:6" s="55" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:6" s="55" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A363" s="55" t="s">
         <v>6</v>
       </c>
@@ -12077,7 +12110,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="364" spans="1:6" s="56" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:6" s="56" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A364" s="56" t="s">
         <v>6</v>
       </c>
@@ -12094,7 +12127,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="365" spans="1:6" s="57" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:6" s="57" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A365" s="57" t="s">
         <v>6</v>
       </c>
@@ -12111,7 +12144,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="366" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:6" ns3:dyDescent="0.3">
       <c r="A366" s="45" t="s">
         <v>6</v>
       </c>
@@ -12129,7 +12162,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="367" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A367" s="45" t="s">
         <v>6</v>
       </c>
@@ -12147,7 +12180,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="368" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:6" ns3:dyDescent="0.3">
       <c r="A368" s="45" t="s">
         <v>6</v>
       </c>
@@ -12161,7 +12194,7 @@
       <c r="E368" s="46"/>
       <c r="F368" s="46"/>
     </row>
-    <row r="369" spans="1:1025" ht="45" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:1025" ht="45" ns3:dyDescent="0.3">
       <c r="A369" s="45" t="s">
         <v>6</v>
       </c>
@@ -12179,7 +12212,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="370" spans="1:1025" ht="30" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:1025" ht="30" ns3:dyDescent="0.3">
       <c r="A370" s="45" t="s">
         <v>6</v>
       </c>
@@ -12197,7 +12230,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="371" spans="1:1025" ht="30" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:1025" ht="30" ns3:dyDescent="0.3">
       <c r="A371" s="45" t="s">
         <v>6</v>
       </c>
@@ -12215,7 +12248,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="372" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A372" s="45" t="s">
         <v>6</v>
       </c>
@@ -12233,7 +12266,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="373" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A373" s="45" t="s">
         <v>6</v>
       </c>
@@ -12247,7 +12280,7 @@
       <c r="E373" s="46"/>
       <c r="F373" s="46"/>
     </row>
-    <row r="374" spans="1:1025" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:1025" s="70" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A374" s="67" t="s">
         <v>6</v>
       </c>
@@ -13284,7 +13317,7 @@
       <c r="AMJ374" s="69"/>
       <c r="AMK374" s="69"/>
     </row>
-    <row r="375" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A375" s="45" t="s">
         <v>6</v>
       </c>
@@ -13302,7 +13335,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="376" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A376" s="45" t="s">
         <v>6</v>
       </c>
@@ -13316,7 +13349,7 @@
       <c r="E376" s="46"/>
       <c r="F376" s="46"/>
     </row>
-    <row r="377" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A377" s="45" t="s">
         <v>6</v>
       </c>
@@ -13334,7 +13367,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="378" spans="1:1025" s="55" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:1025" s="55" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A378" s="55" t="s">
         <v>6</v>
       </c>
@@ -13351,7 +13384,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="379" spans="1:1025" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:1025" s="56" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A379" s="56" t="s">
         <v>6</v>
       </c>
@@ -13368,7 +13401,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="380" spans="1:1025" s="57" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:1025" s="57" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A380" s="57" t="s">
         <v>6</v>
       </c>
@@ -13385,7 +13418,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="381" spans="1:1025" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:1025" ht="15" customHeight="1" ns3:dyDescent="0.3">
       <c r="A381" s="45" t="s">
         <v>6</v>
       </c>
@@ -13403,7 +13436,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="382" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A382" s="45" t="s">
         <v>6</v>
       </c>
@@ -13417,7 +13450,7 @@
       <c r="E382" s="46"/>
       <c r="F382" s="46"/>
     </row>
-    <row r="383" spans="1:1025" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:1025" ns3:dyDescent="0.3">
       <c r="A383" s="45" t="s">
         <v>6</v>
       </c>
@@ -13431,7 +13464,7 @@
       <c r="E383" s="46"/>
       <c r="F383" s="46"/>
     </row>
-    <row r="384" spans="1:1025" ht="60" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:1025" ht="60" ns3:dyDescent="0.3">
       <c r="A384" s="45" t="s">
         <v>6</v>
       </c>
@@ -13449,7 +13482,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="385" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:6" ns3:dyDescent="0.3">
       <c r="A385" s="45" t="s">
         <v>6</v>
       </c>
@@ -13457,17 +13490,17 @@
         <v>740</v>
       </c>
       <c r="C385" s="52" t="s">
-        <v>741</v>
+        <v>1312</v>
       </c>
       <c r="D385" s="45" t="s">
-        <v>742</v>
+        <v>1310</v>
       </c>
       <c r="E385" s="52"/>
       <c r="F385" s="45" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="386" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:6" ns3:dyDescent="0.3">
       <c r="A386" s="45" t="s">
         <v>6</v>
       </c>
@@ -13475,17 +13508,17 @@
         <v>743</v>
       </c>
       <c r="C386" s="52" t="s">
-        <v>744</v>
-      </c>
-      <c r="D386" s="45">
-        <v>78.099999999999994</v>
+        <v>1313</v>
+      </c>
+      <c r="D386" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E386" s="52"/>
       <c r="F386" s="45" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="387" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:6" ns3:dyDescent="0.3">
       <c r="A387" s="45" t="s">
         <v>6</v>
       </c>
@@ -13499,7 +13532,7 @@
       <c r="E387" s="46"/>
       <c r="F387" s="46"/>
     </row>
-    <row r="388" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:6" ns3:dyDescent="0.3">
       <c r="A388" s="45" t="s">
         <v>6</v>
       </c>
@@ -13513,7 +13546,7 @@
       <c r="E388" s="46"/>
       <c r="F388" s="46"/>
     </row>
-    <row r="389" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:6" ns3:dyDescent="0.3">
       <c r="A389" s="45" t="s">
         <v>6</v>
       </c>
@@ -13531,7 +13564,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:6" ns3:dyDescent="0.3">
       <c r="A390" s="45" t="s">
         <v>6</v>
       </c>
@@ -13549,7 +13582,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="391" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:6" ns3:dyDescent="0.3">
       <c r="A391" s="45" t="s">
         <v>6</v>
       </c>
@@ -13567,7 +13600,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="392" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A392" s="45" t="s">
         <v>6</v>
       </c>
@@ -13585,7 +13618,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="393" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A393" s="45" t="s">
         <v>6</v>
       </c>
@@ -13603,7 +13636,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="394" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:6" ns3:dyDescent="0.3">
       <c r="A394" s="45" t="s">
         <v>6</v>
       </c>
@@ -13621,7 +13654,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="395" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A395" s="45" t="s">
         <v>6</v>
       </c>
@@ -13639,7 +13672,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="396" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:6" ns3:dyDescent="0.3">
       <c r="A396" s="45" t="s">
         <v>6</v>
       </c>
@@ -13653,7 +13686,7 @@
       <c r="E396" s="46"/>
       <c r="F396" s="46"/>
     </row>
-    <row r="397" spans="1:6" s="67" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:6" s="67" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A397" s="67" t="s">
         <v>6</v>
       </c>
@@ -13670,7 +13703,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="398" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:6" ns3:dyDescent="0.3">
       <c r="A398" s="45" t="s">
         <v>6</v>
       </c>
@@ -13688,7 +13721,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="399" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:6" ns3:dyDescent="0.3">
       <c r="A399" s="45" t="s">
         <v>6</v>
       </c>
@@ -13702,7 +13735,7 @@
       <c r="E399" s="46"/>
       <c r="F399" s="46"/>
     </row>
-    <row r="400" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:6" ns3:dyDescent="0.3">
       <c r="A400" s="45" t="s">
         <v>6</v>
       </c>
@@ -13720,7 +13753,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="401" spans="1:6" s="55" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:6" s="55" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A401" s="55" t="s">
         <v>6</v>
       </c>
@@ -13737,7 +13770,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="402" spans="1:6" s="56" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:6" s="56" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A402" s="56" t="s">
         <v>6</v>
       </c>
@@ -13754,7 +13787,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="403" spans="1:6" s="57" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:6" s="57" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A403" s="57" t="s">
         <v>6</v>
       </c>
@@ -13771,7 +13804,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="404" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:6" ns3:dyDescent="0.3">
       <c r="A404" s="45" t="s">
         <v>6</v>
       </c>
@@ -13789,7 +13822,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="405" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:6" ns3:dyDescent="0.3">
       <c r="A405" s="45" t="s">
         <v>6</v>
       </c>
@@ -13803,7 +13836,7 @@
       <c r="E405" s="46"/>
       <c r="F405" s="46"/>
     </row>
-    <row r="406" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:6" ns3:dyDescent="0.3">
       <c r="A406" s="45" t="s">
         <v>6</v>
       </c>
@@ -13817,7 +13850,7 @@
       <c r="E406" s="46"/>
       <c r="F406" s="46"/>
     </row>
-    <row r="407" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:6" ht="60" ns3:dyDescent="0.3">
       <c r="A407" s="45" t="s">
         <v>6</v>
       </c>
@@ -13835,7 +13868,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="408" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:6" ns3:dyDescent="0.3">
       <c r="A408" s="45" t="s">
         <v>6</v>
       </c>
@@ -13843,17 +13876,17 @@
         <v>774</v>
       </c>
       <c r="C408" s="45" t="s">
-        <v>775</v>
+        <v>1314</v>
       </c>
       <c r="D408" s="45" t="s">
-        <v>742</v>
+        <v>1310</v>
       </c>
       <c r="E408" s="45"/>
       <c r="F408" s="45" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="409" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:6" ns3:dyDescent="0.3">
       <c r="A409" s="45" t="s">
         <v>6</v>
       </c>
@@ -13861,17 +13894,17 @@
         <v>776</v>
       </c>
       <c r="C409" s="52" t="s">
-        <v>777</v>
-      </c>
-      <c r="D409" s="45">
-        <v>78.099999999999994</v>
+        <v>1315</v>
+      </c>
+      <c r="D409" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E409" s="52"/>
       <c r="F409" s="45" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="410" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:6" ns3:dyDescent="0.3">
       <c r="A410" s="45" t="s">
         <v>6</v>
       </c>
@@ -13885,7 +13918,7 @@
       <c r="E410" s="46"/>
       <c r="F410" s="46"/>
     </row>
-    <row r="411" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:6" ns3:dyDescent="0.3">
       <c r="A411" s="45" t="s">
         <v>6</v>
       </c>
@@ -13899,7 +13932,7 @@
       <c r="E411" s="46"/>
       <c r="F411" s="46"/>
     </row>
-    <row r="412" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:6" ns3:dyDescent="0.3">
       <c r="A412" s="45" t="s">
         <v>6</v>
       </c>
@@ -13917,7 +13950,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:6" ns3:dyDescent="0.3">
       <c r="A413" s="45" t="s">
         <v>6</v>
       </c>
@@ -13935,7 +13968,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="414" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:6" ns3:dyDescent="0.3">
       <c r="A414" s="45" t="s">
         <v>6</v>
       </c>
@@ -13953,7 +13986,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="415" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:6" ns3:dyDescent="0.3">
       <c r="A415" s="45" t="s">
         <v>6</v>
       </c>
@@ -13971,7 +14004,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="416" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A416" s="45" t="s">
         <v>6</v>
       </c>
@@ -13989,7 +14022,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="417" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:6" ns3:dyDescent="0.3">
       <c r="A417" s="45" t="s">
         <v>6</v>
       </c>
@@ -14007,7 +14040,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="418" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A418" s="45" t="s">
         <v>6</v>
       </c>
@@ -14025,7 +14058,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="419" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:6" ns3:dyDescent="0.3">
       <c r="A419" s="45" t="s">
         <v>6</v>
       </c>
@@ -14039,7 +14072,7 @@
       <c r="E419" s="46"/>
       <c r="F419" s="46"/>
     </row>
-    <row r="420" spans="1:6" s="67" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:6" s="67" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A420" s="67" t="s">
         <v>6</v>
       </c>
@@ -14056,7 +14089,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="421" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:6" ns3:dyDescent="0.3">
       <c r="A421" s="45" t="s">
         <v>6</v>
       </c>
@@ -14074,7 +14107,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="422" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:6" ns3:dyDescent="0.3">
       <c r="A422" s="45" t="s">
         <v>6</v>
       </c>
@@ -14088,7 +14121,7 @@
       <c r="E422" s="46"/>
       <c r="F422" s="46"/>
     </row>
-    <row r="423" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:6" ns3:dyDescent="0.3">
       <c r="A423" s="45" t="s">
         <v>6</v>
       </c>
@@ -14106,7 +14139,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="424" spans="1:6" s="55" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:6" s="55" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A424" s="55" t="s">
         <v>6</v>
       </c>
@@ -14123,7 +14156,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="425" spans="1:6" s="56" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:6" s="56" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A425" s="56" t="s">
         <v>6</v>
       </c>
@@ -14140,7 +14173,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="426" spans="1:6" s="57" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:6" s="57" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A426" s="57" t="s">
         <v>6</v>
       </c>
@@ -14157,7 +14190,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="427" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:6" ns3:dyDescent="0.3">
       <c r="A427" s="45" t="s">
         <v>6</v>
       </c>
@@ -14175,7 +14208,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="428" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:6" ns3:dyDescent="0.3">
       <c r="A428" s="45" t="s">
         <v>6</v>
       </c>
@@ -14189,7 +14222,7 @@
       <c r="E428" s="46"/>
       <c r="F428" s="46"/>
     </row>
-    <row r="429" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:6" ns3:dyDescent="0.3">
       <c r="A429" s="45" t="s">
         <v>6</v>
       </c>
@@ -14203,7 +14236,7 @@
       <c r="E429" s="46"/>
       <c r="F429" s="46"/>
     </row>
-    <row r="430" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:6" ht="60" ns3:dyDescent="0.3">
       <c r="A430" s="45" t="s">
         <v>6</v>
       </c>
@@ -14221,7 +14254,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="431" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:6" ns3:dyDescent="0.3">
       <c r="A431" s="45" t="s">
         <v>6</v>
       </c>
@@ -14229,17 +14262,17 @@
         <v>804</v>
       </c>
       <c r="C431" s="52" t="s">
-        <v>805</v>
-      </c>
-      <c r="D431" s="45">
-        <v>78.099999999999994</v>
+        <v>1316</v>
+      </c>
+      <c r="D431" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E431" s="52"/>
       <c r="F431" s="45" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="432" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:6" ns3:dyDescent="0.3">
       <c r="A432" s="45" t="s">
         <v>6</v>
       </c>
@@ -14247,17 +14280,17 @@
         <v>806</v>
       </c>
       <c r="C432" s="52" t="s">
-        <v>777</v>
-      </c>
-      <c r="D432" s="45">
-        <v>78.099999999999994</v>
+        <v>1317</v>
+      </c>
+      <c r="D432" s="45" t="s">
+        <v>1310</v>
       </c>
       <c r="E432" s="52"/>
       <c r="F432" s="45" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="433" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:6" ns3:dyDescent="0.3">
       <c r="A433" s="45" t="s">
         <v>6</v>
       </c>
@@ -14271,7 +14304,7 @@
       <c r="E433" s="46"/>
       <c r="F433" s="46"/>
     </row>
-    <row r="434" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:6" ns3:dyDescent="0.3">
       <c r="A434" s="45" t="s">
         <v>6</v>
       </c>
@@ -14285,7 +14318,7 @@
       <c r="E434" s="46"/>
       <c r="F434" s="46"/>
     </row>
-    <row r="435" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:6" ns3:dyDescent="0.3">
       <c r="A435" s="45" t="s">
         <v>6</v>
       </c>
@@ -14303,7 +14336,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="436" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:6" ns3:dyDescent="0.3">
       <c r="A436" s="45" t="s">
         <v>6</v>
       </c>
@@ -14321,7 +14354,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="437" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:6" ns3:dyDescent="0.3">
       <c r="A437" s="45" t="s">
         <v>6</v>
       </c>
@@ -14339,7 +14372,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="438" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:6" ns3:dyDescent="0.3">
       <c r="A438" s="45" t="s">
         <v>6</v>
       </c>
@@ -14357,7 +14390,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="439" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:6" ns3:dyDescent="0.3">
       <c r="A439" s="45" t="s">
         <v>6</v>
       </c>
@@ -14371,7 +14404,7 @@
       <c r="E439" s="46"/>
       <c r="F439" s="46"/>
     </row>
-    <row r="440" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:6" ns3:dyDescent="0.3">
       <c r="A440" s="45" t="s">
         <v>6</v>
       </c>
@@ -14389,7 +14422,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="441" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:6" ns3:dyDescent="0.3">
       <c r="A441" s="45" t="s">
         <v>6</v>
       </c>
@@ -14407,7 +14440,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="442" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:6" ns3:dyDescent="0.3">
       <c r="A442" s="45" t="s">
         <v>6</v>
       </c>
@@ -14425,7 +14458,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="443" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:6" ns3:dyDescent="0.3">
       <c r="A443" s="45" t="s">
         <v>6</v>
       </c>
@@ -14439,7 +14472,7 @@
       <c r="E443" s="46"/>
       <c r="F443" s="46"/>
     </row>
-    <row r="444" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:6" ns3:dyDescent="0.3">
       <c r="A444" s="45" t="s">
         <v>6</v>
       </c>
@@ -14457,7 +14490,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="445" spans="1:6" s="55" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:6" s="55" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A445" s="55" t="s">
         <v>6</v>
       </c>
@@ -14474,7 +14507,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="446" spans="1:6" s="56" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:6" s="56" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A446" s="56" t="s">
         <v>6</v>
       </c>
@@ -14491,7 +14524,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="447" spans="1:6" s="57" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:6" s="57" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A447" s="57" t="s">
         <v>6</v>
       </c>
@@ -14508,7 +14541,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="448" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:6" ns3:dyDescent="0.3">
       <c r="A448" s="45" t="s">
         <v>6</v>
       </c>
@@ -14526,7 +14559,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="449" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A449" s="45" t="s">
         <v>6</v>
       </c>
@@ -14544,7 +14577,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="450" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:6" ns3:dyDescent="0.3">
       <c r="A450" s="45" t="s">
         <v>6</v>
       </c>
@@ -14558,7 +14591,7 @@
       <c r="E450" s="46"/>
       <c r="F450" s="46"/>
     </row>
-    <row r="451" spans="1:6" ht="45" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:6" ht="45" ns3:dyDescent="0.3">
       <c r="A451" s="45" t="s">
         <v>6</v>
       </c>
@@ -14576,7 +14609,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="452" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A452" s="45" t="s">
         <v>6</v>
       </c>
@@ -14594,7 +14627,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="453" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:6" ns3:dyDescent="0.3">
       <c r="A453" s="45" t="s">
         <v>6</v>
       </c>
@@ -14612,7 +14645,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="454" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:6" ns3:dyDescent="0.3">
       <c r="A454" s="45" t="s">
         <v>6</v>
       </c>
@@ -14630,7 +14663,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="455" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:6" ns3:dyDescent="0.3">
       <c r="A455" s="45" t="s">
         <v>6</v>
       </c>
@@ -14644,7 +14677,7 @@
       <c r="E455" s="46"/>
       <c r="F455" s="46"/>
     </row>
-    <row r="456" spans="1:6" s="67" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:6" s="67" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A456" s="67" t="s">
         <v>6</v>
       </c>
@@ -14661,7 +14694,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="457" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:6" ns3:dyDescent="0.3">
       <c r="A457" s="45" t="s">
         <v>6</v>
       </c>
@@ -14679,7 +14712,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="458" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:6" ns3:dyDescent="0.3">
       <c r="A458" s="45" t="s">
         <v>6</v>
       </c>
@@ -14693,7 +14726,7 @@
       <c r="E458" s="46"/>
       <c r="F458" s="46"/>
     </row>
-    <row r="459" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:6" ns3:dyDescent="0.3">
       <c r="A459" s="45" t="s">
         <v>6</v>
       </c>
@@ -14711,7 +14744,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="460" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A460" s="45" t="s">
         <v>6</v>
       </c>
@@ -14725,7 +14758,7 @@
       <c r="E460" s="44"/>
       <c r="F460" s="46"/>
     </row>
-    <row r="461" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:6" ns3:dyDescent="0.3">
       <c r="A461" s="45" t="s">
         <v>6</v>
       </c>
@@ -14739,7 +14772,7 @@
       <c r="E461" s="52"/>
       <c r="F461" s="45"/>
     </row>
-    <row r="462" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:6" ns3:dyDescent="0.3">
       <c r="A462" s="45" t="s">
         <v>6</v>
       </c>
@@ -14753,7 +14786,7 @@
       <c r="E462" s="52"/>
       <c r="F462" s="45"/>
     </row>
-    <row r="463" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:6" ns3:dyDescent="0.3">
       <c r="A463" s="45" t="s">
         <v>6</v>
       </c>
@@ -14767,7 +14800,7 @@
       <c r="E463" s="52"/>
       <c r="F463" s="45"/>
     </row>
-    <row r="464" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:6" ns3:dyDescent="0.3">
       <c r="A464" s="45" t="s">
         <v>6</v>
       </c>
@@ -14781,7 +14814,7 @@
       <c r="E464" s="44"/>
       <c r="F464" s="46"/>
     </row>
-    <row r="465" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:6" ns3:dyDescent="0.3">
       <c r="A465" s="45" t="s">
         <v>6</v>
       </c>
@@ -14795,7 +14828,7 @@
       <c r="E465" s="52"/>
       <c r="F465" s="45"/>
     </row>
-    <row r="466" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:6" ns3:dyDescent="0.3">
       <c r="A466" s="45" t="s">
         <v>6</v>
       </c>
@@ -14809,7 +14842,7 @@
       <c r="E466" s="52"/>
       <c r="F466" s="45"/>
     </row>
-    <row r="467" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:6" ns3:dyDescent="0.3">
       <c r="A467" s="45" t="s">
         <v>6</v>
       </c>
@@ -14823,7 +14856,7 @@
       <c r="E467" s="44"/>
       <c r="F467" s="46"/>
     </row>
-    <row r="468" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:6" ns3:dyDescent="0.3">
       <c r="A468" s="45" t="s">
         <v>6</v>
       </c>
@@ -14837,7 +14870,7 @@
       <c r="E468" s="46"/>
       <c r="F468" s="46"/>
     </row>
-    <row r="469" spans="1:6" ht="60" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:6" ht="60" ns3:dyDescent="0.3">
       <c r="A469" s="45" t="s">
         <v>6</v>
       </c>
@@ -14855,7 +14888,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="470" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:6" ns3:dyDescent="0.3">
       <c r="A470" s="45" t="s">
         <v>6</v>
       </c>
@@ -14873,7 +14906,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="471" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:6" ns3:dyDescent="0.3">
       <c r="A471" s="45" t="s">
         <v>6</v>
       </c>
@@ -14891,7 +14924,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="472" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:6" ns3:dyDescent="0.3">
       <c r="A472" s="45" t="s">
         <v>6</v>
       </c>
@@ -14905,7 +14938,7 @@
       <c r="E472" s="46"/>
       <c r="F472" s="46"/>
     </row>
-    <row r="473" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:6" ns3:dyDescent="0.3">
       <c r="A473" s="45" t="s">
         <v>6</v>
       </c>
@@ -14919,7 +14952,7 @@
       <c r="E473" s="46"/>
       <c r="F473" s="46"/>
     </row>
-    <row r="474" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:6" ns3:dyDescent="0.3">
       <c r="A474" s="45" t="s">
         <v>6</v>
       </c>
@@ -14937,7 +14970,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="475" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:6" ns3:dyDescent="0.3">
       <c r="A475" s="45" t="s">
         <v>6</v>
       </c>
@@ -14955,7 +14988,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="476" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:6" ns3:dyDescent="0.3">
       <c r="A476" s="45" t="s">
         <v>6</v>
       </c>
@@ -14973,7 +15006,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="477" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:6" ns3:dyDescent="0.3">
       <c r="A477" s="45" t="s">
         <v>6</v>
       </c>
@@ -14991,7 +15024,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="478" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A478" s="45" t="s">
         <v>6</v>
       </c>
@@ -15009,7 +15042,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="479" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:6" ns3:dyDescent="0.3">
       <c r="A479" s="45" t="s">
         <v>6</v>
       </c>
@@ -15025,7 +15058,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="480" spans="1:6" ht="30" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:6" ht="30" ns3:dyDescent="0.3">
       <c r="A480" s="45" t="s">
         <v>6</v>
       </c>
@@ -15043,7 +15076,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="481" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:6" ns3:dyDescent="0.3">
       <c r="A481" s="45" t="s">
         <v>6</v>
       </c>
@@ -15061,7 +15094,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="482" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:6" ns3:dyDescent="0.3">
       <c r="A482" s="45" t="s">
         <v>6</v>
       </c>
@@ -15075,7 +15108,7 @@
       <c r="E482" s="46"/>
       <c r="F482" s="46"/>
     </row>
-    <row r="483" spans="1:6" s="67" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:6" s="67" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A483" s="67" t="s">
         <v>6</v>
       </c>
@@ -15092,7 +15125,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="484" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:6" ns3:dyDescent="0.3">
       <c r="A484" s="45" t="s">
         <v>6</v>
       </c>
@@ -15110,7 +15143,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="485" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:6" ns3:dyDescent="0.3">
       <c r="A485" s="45" t="s">
         <v>6</v>
       </c>
@@ -15124,7 +15157,7 @@
       <c r="E485" s="46"/>
       <c r="F485" s="46"/>
     </row>
-    <row r="486" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:6" ns3:dyDescent="0.3">
       <c r="A486" s="45" t="s">
         <v>6</v>
       </c>
@@ -15142,7 +15175,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="487" spans="1:6" s="55" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:6" s="55" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A487" s="55" t="s">
         <v>6</v>
       </c>
@@ -15159,7 +15192,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="488" spans="1:6" s="56" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="488" spans="1:6" s="56" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A488" s="56" t="s">
         <v>6</v>
       </c>
@@ -15176,7 +15209,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="489" spans="1:6" s="57" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:6" s="57" customFormat="1" ht="15" ns3:dyDescent="0.3">
       <c r="A489" s="57" t="s">
         <v>6</v>
       </c>
@@ -15193,7 +15226,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="490" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:6" ns3:dyDescent="0.3">
       <c r="A490" s="45" t="s">
         <v>6</v>
       </c>
@@ -15212,7 +15245,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D485" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="D1:D485" ns2:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
         <filter val="PKIX.13"/>
@@ -15220,7 +15253,7 @@
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" ns4:id="rId1"/>
 </worksheet>
 </file>
 
@@ -18805,9 +18838,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AMK4"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.8984375" style="8" customWidth="1"/>
     <col min="2" max="2" width="54.59765625" style="8" customWidth="1"/>
@@ -18819,7 +18852,7 @@
     <col min="257" max="1025" width="8.8984375" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:256" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:256" ns3:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>888</v>
       </c>
@@ -18842,7 +18875,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="2" spans="1:256" s="32" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:256" s="32" customFormat="1" ht="31.2" ns3:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>742</v>
       </c>
@@ -19110,7 +19143,7 @@
       <c r="IU2" s="31"/>
       <c r="IV2" s="31"/>
     </row>
-    <row r="3" spans="1:256" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:256" ht="31.2" ns3:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>1186</v>
       </c>
@@ -19129,7 +19162,7 @@
       </c>
       <c r="G3" s="11"/>
     </row>
-    <row r="4" spans="1:256" ht="78" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:256" ht="78" ns3:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>739</v>
       </c>
@@ -19147,6 +19180,274 @@
         <v>897</v>
       </c>
       <c r="G4" s="11"/>
+    </row>
+    <row r="5" spans="1:256" s="32" customFormat="1" ht="31.2" ns3:dyDescent="0.3">
+      <c r="A5" s="33" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>1318</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>1319</v>
+      </c>
+      <c r="E5" s="23"/>
+      <c r="F5" s="12" t="s">
+        <v>897</v>
+      </c>
+      <c r="G5" s="12"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+      <c r="Y5" s="31"/>
+      <c r="Z5" s="31"/>
+      <c r="AA5" s="31"/>
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="31"/>
+      <c r="AD5" s="31"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="31"/>
+      <c r="AG5" s="31"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="31"/>
+      <c r="AJ5" s="31"/>
+      <c r="AK5" s="31"/>
+      <c r="AL5" s="31"/>
+      <c r="AM5" s="31"/>
+      <c r="AN5" s="31"/>
+      <c r="AO5" s="31"/>
+      <c r="AP5" s="31"/>
+      <c r="AQ5" s="31"/>
+      <c r="AR5" s="31"/>
+      <c r="AS5" s="31"/>
+      <c r="AT5" s="31"/>
+      <c r="AU5" s="31"/>
+      <c r="AV5" s="31"/>
+      <c r="AW5" s="31"/>
+      <c r="AX5" s="31"/>
+      <c r="AY5" s="31"/>
+      <c r="AZ5" s="31"/>
+      <c r="BA5" s="31"/>
+      <c r="BB5" s="31"/>
+      <c r="BC5" s="31"/>
+      <c r="BD5" s="31"/>
+      <c r="BE5" s="31"/>
+      <c r="BF5" s="31"/>
+      <c r="BG5" s="31"/>
+      <c r="BH5" s="31"/>
+      <c r="BI5" s="31"/>
+      <c r="BJ5" s="31"/>
+      <c r="BK5" s="31"/>
+      <c r="BL5" s="31"/>
+      <c r="BM5" s="31"/>
+      <c r="BN5" s="31"/>
+      <c r="BO5" s="31"/>
+      <c r="BP5" s="31"/>
+      <c r="BQ5" s="31"/>
+      <c r="BR5" s="31"/>
+      <c r="BS5" s="31"/>
+      <c r="BT5" s="31"/>
+      <c r="BU5" s="31"/>
+      <c r="BV5" s="31"/>
+      <c r="BW5" s="31"/>
+      <c r="BX5" s="31"/>
+      <c r="BY5" s="31"/>
+      <c r="BZ5" s="31"/>
+      <c r="CA5" s="31"/>
+      <c r="CB5" s="31"/>
+      <c r="CC5" s="31"/>
+      <c r="CD5" s="31"/>
+      <c r="CE5" s="31"/>
+      <c r="CF5" s="31"/>
+      <c r="CG5" s="31"/>
+      <c r="CH5" s="31"/>
+      <c r="CI5" s="31"/>
+      <c r="CJ5" s="31"/>
+      <c r="CK5" s="31"/>
+      <c r="CL5" s="31"/>
+      <c r="CM5" s="31"/>
+      <c r="CN5" s="31"/>
+      <c r="CO5" s="31"/>
+      <c r="CP5" s="31"/>
+      <c r="CQ5" s="31"/>
+      <c r="CR5" s="31"/>
+      <c r="CS5" s="31"/>
+      <c r="CT5" s="31"/>
+      <c r="CU5" s="31"/>
+      <c r="CV5" s="31"/>
+      <c r="CW5" s="31"/>
+      <c r="CX5" s="31"/>
+      <c r="CY5" s="31"/>
+      <c r="CZ5" s="31"/>
+      <c r="DA5" s="31"/>
+      <c r="DB5" s="31"/>
+      <c r="DC5" s="31"/>
+      <c r="DD5" s="31"/>
+      <c r="DE5" s="31"/>
+      <c r="DF5" s="31"/>
+      <c r="DG5" s="31"/>
+      <c r="DH5" s="31"/>
+      <c r="DI5" s="31"/>
+      <c r="DJ5" s="31"/>
+      <c r="DK5" s="31"/>
+      <c r="DL5" s="31"/>
+      <c r="DM5" s="31"/>
+      <c r="DN5" s="31"/>
+      <c r="DO5" s="31"/>
+      <c r="DP5" s="31"/>
+      <c r="DQ5" s="31"/>
+      <c r="DR5" s="31"/>
+      <c r="DS5" s="31"/>
+      <c r="DT5" s="31"/>
+      <c r="DU5" s="31"/>
+      <c r="DV5" s="31"/>
+      <c r="DW5" s="31"/>
+      <c r="DX5" s="31"/>
+      <c r="DY5" s="31"/>
+      <c r="DZ5" s="31"/>
+      <c r="EA5" s="31"/>
+      <c r="EB5" s="31"/>
+      <c r="EC5" s="31"/>
+      <c r="ED5" s="31"/>
+      <c r="EE5" s="31"/>
+      <c r="EF5" s="31"/>
+      <c r="EG5" s="31"/>
+      <c r="EH5" s="31"/>
+      <c r="EI5" s="31"/>
+      <c r="EJ5" s="31"/>
+      <c r="EK5" s="31"/>
+      <c r="EL5" s="31"/>
+      <c r="EM5" s="31"/>
+      <c r="EN5" s="31"/>
+      <c r="EO5" s="31"/>
+      <c r="EP5" s="31"/>
+      <c r="EQ5" s="31"/>
+      <c r="ER5" s="31"/>
+      <c r="ES5" s="31"/>
+      <c r="ET5" s="31"/>
+      <c r="EU5" s="31"/>
+      <c r="EV5" s="31"/>
+      <c r="EW5" s="31"/>
+      <c r="EX5" s="31"/>
+      <c r="EY5" s="31"/>
+      <c r="EZ5" s="31"/>
+      <c r="FA5" s="31"/>
+      <c r="FB5" s="31"/>
+      <c r="FC5" s="31"/>
+      <c r="FD5" s="31"/>
+      <c r="FE5" s="31"/>
+      <c r="FF5" s="31"/>
+      <c r="FG5" s="31"/>
+      <c r="FH5" s="31"/>
+      <c r="FI5" s="31"/>
+      <c r="FJ5" s="31"/>
+      <c r="FK5" s="31"/>
+      <c r="FL5" s="31"/>
+      <c r="FM5" s="31"/>
+      <c r="FN5" s="31"/>
+      <c r="FO5" s="31"/>
+      <c r="FP5" s="31"/>
+      <c r="FQ5" s="31"/>
+      <c r="FR5" s="31"/>
+      <c r="FS5" s="31"/>
+      <c r="FT5" s="31"/>
+      <c r="FU5" s="31"/>
+      <c r="FV5" s="31"/>
+      <c r="FW5" s="31"/>
+      <c r="FX5" s="31"/>
+      <c r="FY5" s="31"/>
+      <c r="FZ5" s="31"/>
+      <c r="GA5" s="31"/>
+      <c r="GB5" s="31"/>
+      <c r="GC5" s="31"/>
+      <c r="GD5" s="31"/>
+      <c r="GE5" s="31"/>
+      <c r="GF5" s="31"/>
+      <c r="GG5" s="31"/>
+      <c r="GH5" s="31"/>
+      <c r="GI5" s="31"/>
+      <c r="GJ5" s="31"/>
+      <c r="GK5" s="31"/>
+      <c r="GL5" s="31"/>
+      <c r="GM5" s="31"/>
+      <c r="GN5" s="31"/>
+      <c r="GO5" s="31"/>
+      <c r="GP5" s="31"/>
+      <c r="GQ5" s="31"/>
+      <c r="GR5" s="31"/>
+      <c r="GS5" s="31"/>
+      <c r="GT5" s="31"/>
+      <c r="GU5" s="31"/>
+      <c r="GV5" s="31"/>
+      <c r="GW5" s="31"/>
+      <c r="GX5" s="31"/>
+      <c r="GY5" s="31"/>
+      <c r="GZ5" s="31"/>
+      <c r="HA5" s="31"/>
+      <c r="HB5" s="31"/>
+      <c r="HC5" s="31"/>
+      <c r="HD5" s="31"/>
+      <c r="HE5" s="31"/>
+      <c r="HF5" s="31"/>
+      <c r="HG5" s="31"/>
+      <c r="HH5" s="31"/>
+      <c r="HI5" s="31"/>
+      <c r="HJ5" s="31"/>
+      <c r="HK5" s="31"/>
+      <c r="HL5" s="31"/>
+      <c r="HM5" s="31"/>
+      <c r="HN5" s="31"/>
+      <c r="HO5" s="31"/>
+      <c r="HP5" s="31"/>
+      <c r="HQ5" s="31"/>
+      <c r="HR5" s="31"/>
+      <c r="HS5" s="31"/>
+      <c r="HT5" s="31"/>
+      <c r="HU5" s="31"/>
+      <c r="HV5" s="31"/>
+      <c r="HW5" s="31"/>
+      <c r="HX5" s="31"/>
+      <c r="HY5" s="31"/>
+      <c r="HZ5" s="31"/>
+      <c r="IA5" s="31"/>
+      <c r="IB5" s="31"/>
+      <c r="IC5" s="31"/>
+      <c r="ID5" s="31"/>
+      <c r="IE5" s="31"/>
+      <c r="IF5" s="31"/>
+      <c r="IG5" s="31"/>
+      <c r="IH5" s="31"/>
+      <c r="II5" s="31"/>
+      <c r="IJ5" s="31"/>
+      <c r="IK5" s="31"/>
+      <c r="IL5" s="31"/>
+      <c r="IM5" s="31"/>
+      <c r="IN5" s="31"/>
+      <c r="IO5" s="31"/>
+      <c r="IP5" s="31"/>
+      <c r="IQ5" s="31"/>
+      <c r="IR5" s="31"/>
+      <c r="IS5" s="31"/>
+      <c r="IT5" s="31"/>
+      <c r="IU5" s="31"/>
+      <c r="IV5" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
Apply SP 800-73-5 CCC eliminated-tag check in PIV profiles
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1320" uniqueCount="1320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1324">
   <si>
     <t>Document</t>
   </si>
@@ -3995,6 +3995,18 @@
   </si>
   <si>
     <t>Validate active PIV certificate public-key algorithms, sizes, curves, and RSA exponent against SP 800-78-5 Section 3.1, Table 1 (through 2030).</t>
+  </si>
+  <si>
+    <t>CCC eliminated optional tags E3 and B4 are absent under SP 800-73-5 Part 1 Appendix A Table 9.</t>
+  </si>
+  <si>
+    <t>73-5.4.current</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_4</t>
+  </si>
+  <si>
+    <t>Reject eliminated CCC tags E3 and B4 under SP 800-73-5 Part 1 Appendix A Table 9.</t>
   </si>
 </sst>
 </file>
@@ -5030,10 +5042,10 @@
         <v>35</v>
       </c>
       <c r="C12" s="45" t="s">
-        <v>36</v>
+        <v>1320</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>37</v>
+        <v>1321</v>
       </c>
       <c r="E12" s="45"/>
       <c r="F12" s="45" t="s">
@@ -15398,9 +15410,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMK56"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:AMK57"/>
+  <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" style="13" customWidth="1"/>
     <col min="2" max="2" width="88.296875" style="8" customWidth="1"/>
@@ -15412,7 +15424,7 @@
     <col min="8" max="1025" width="8.8984375" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="18" customFormat="1" ns3:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>888</v>
       </c>
@@ -15435,7 +15447,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ns3:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>28</v>
       </c>
@@ -15454,7 +15466,7 @@
       </c>
       <c r="G2" s="17"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ns3:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>31</v>
       </c>
@@ -15473,7 +15485,7 @@
       </c>
       <c r="G3" s="17"/>
     </row>
-    <row r="4" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>34</v>
       </c>
@@ -15492,7 +15504,7 @@
       </c>
       <c r="G4" s="17"/>
     </row>
-    <row r="5" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>37</v>
       </c>
@@ -15511,7 +15523,7 @@
       </c>
       <c r="G5" s="17"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ns3:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>40</v>
       </c>
@@ -15530,7 +15542,7 @@
       </c>
       <c r="G6" s="17"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ns3:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>46</v>
       </c>
@@ -15549,7 +15561,7 @@
       </c>
       <c r="G7" s="17"/>
     </row>
-    <row r="8" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>913</v>
       </c>
@@ -15568,7 +15580,7 @@
       </c>
       <c r="G8" s="17"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ns3:dyDescent="0.3">
       <c r="A9" s="16" t="s">
         <v>57</v>
       </c>
@@ -15587,7 +15599,7 @@
       </c>
       <c r="G9" s="17"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ns3:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>99</v>
       </c>
@@ -15606,7 +15618,7 @@
       </c>
       <c r="G10" s="17"/>
     </row>
-    <row r="11" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>60</v>
       </c>
@@ -15625,7 +15637,7 @@
       </c>
       <c r="G11" s="17"/>
     </row>
-    <row r="12" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A12" s="16" t="s">
         <v>66</v>
       </c>
@@ -15644,7 +15656,7 @@
       </c>
       <c r="G12" s="17"/>
     </row>
-    <row r="13" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="78" ns3:dyDescent="0.3">
       <c r="A13" s="19" t="s">
         <v>105</v>
       </c>
@@ -15663,7 +15675,7 @@
       </c>
       <c r="G13" s="17"/>
     </row>
-    <row r="14" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A14" s="16" t="s">
         <v>81</v>
       </c>
@@ -15682,7 +15694,7 @@
       </c>
       <c r="G14" s="17"/>
     </row>
-    <row r="15" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A15" s="16" t="s">
         <v>84</v>
       </c>
@@ -15701,7 +15713,7 @@
       </c>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ns3:dyDescent="0.3">
       <c r="A16" s="16" t="s">
         <v>108</v>
       </c>
@@ -15720,7 +15732,7 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ns3:dyDescent="0.3">
       <c r="A17" s="16" t="s">
         <v>111</v>
       </c>
@@ -15741,7 +15753,7 @@
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A18" s="16" t="s">
         <v>102</v>
       </c>
@@ -15760,7 +15772,7 @@
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="46.8" ns3:dyDescent="0.3">
       <c r="A19" s="15" t="s">
         <v>931</v>
       </c>
@@ -15779,7 +15791,7 @@
       </c>
       <c r="G19" s="19"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ns3:dyDescent="0.3">
       <c r="A20" s="16" t="s">
         <v>132</v>
       </c>
@@ -15798,7 +15810,7 @@
       </c>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" ns3:dyDescent="0.3">
       <c r="A21" s="16" t="s">
         <v>135</v>
       </c>
@@ -15817,7 +15829,7 @@
       </c>
       <c r="G21" s="17"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" ns3:dyDescent="0.3">
       <c r="A22" s="16" t="s">
         <v>138</v>
       </c>
@@ -15836,7 +15848,7 @@
       </c>
       <c r="G22" s="17"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" ns3:dyDescent="0.3">
       <c r="A23" s="16" t="s">
         <v>141</v>
       </c>
@@ -15855,7 +15867,7 @@
       </c>
       <c r="G23" s="17"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" ns3:dyDescent="0.3">
       <c r="A24" s="16" t="s">
         <v>43</v>
       </c>
@@ -15874,7 +15886,7 @@
       </c>
       <c r="G24" s="17"/>
     </row>
-    <row r="25" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A25" s="16" t="s">
         <v>116</v>
       </c>
@@ -15893,7 +15905,7 @@
       </c>
       <c r="G25" s="17"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ns3:dyDescent="0.3">
       <c r="A26" s="16" t="s">
         <v>195</v>
       </c>
@@ -15912,7 +15924,7 @@
       </c>
       <c r="G26" s="17"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" ns3:dyDescent="0.3">
       <c r="A27" s="16" t="s">
         <v>198</v>
       </c>
@@ -15931,7 +15943,7 @@
       </c>
       <c r="G27" s="17"/>
     </row>
-    <row r="28" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A28" s="16" t="s">
         <v>164</v>
       </c>
@@ -15950,7 +15962,7 @@
       </c>
       <c r="G28" s="17"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" ns3:dyDescent="0.3">
       <c r="A29" s="16" t="s">
         <v>167</v>
       </c>
@@ -15969,7 +15981,7 @@
       </c>
       <c r="G29" s="17"/>
     </row>
-    <row r="30" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A30" s="16" t="s">
         <v>176</v>
       </c>
@@ -15988,7 +16000,7 @@
       </c>
       <c r="G30" s="17"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" ns3:dyDescent="0.3">
       <c r="A31" s="16" t="s">
         <v>179</v>
       </c>
@@ -16007,7 +16019,7 @@
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" ht="30" ns3:dyDescent="0.3">
       <c r="A32" s="16" t="s">
         <v>181</v>
       </c>
@@ -16026,7 +16038,7 @@
       </c>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A33" s="16" t="s">
         <v>192</v>
       </c>
@@ -16045,7 +16057,7 @@
       </c>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A34" s="16" t="s">
         <v>251</v>
       </c>
@@ -16064,7 +16076,7 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" ns3:dyDescent="0.3">
       <c r="A35" s="16" t="s">
         <v>254</v>
       </c>
@@ -16083,7 +16095,7 @@
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" ns3:dyDescent="0.3">
       <c r="A36" s="16" t="s">
         <v>260</v>
       </c>
@@ -16102,7 +16114,7 @@
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A37" s="16" t="s">
         <v>263</v>
       </c>
@@ -16121,7 +16133,7 @@
       </c>
       <c r="G37" s="19"/>
     </row>
-    <row r="38" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" ht="46.8" ns3:dyDescent="0.3">
       <c r="A38" s="16" t="s">
         <v>618</v>
       </c>
@@ -16140,7 +16152,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A39" s="16" t="s">
         <v>289</v>
       </c>
@@ -16159,7 +16171,7 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ns3:dyDescent="0.3">
       <c r="A40" s="16" t="s">
         <v>274</v>
       </c>
@@ -16178,7 +16190,7 @@
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" ns3:dyDescent="0.3">
       <c r="A41" s="16" t="s">
         <v>277</v>
       </c>
@@ -16197,7 +16209,7 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" ht="78" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="78" ns3:dyDescent="0.3">
       <c r="A42" s="16" t="s">
         <v>286</v>
       </c>
@@ -16216,7 +16228,7 @@
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" ns3:dyDescent="0.3">
       <c r="A43" s="20" t="s">
         <v>63</v>
       </c>
@@ -16235,7 +16247,7 @@
       </c>
       <c r="G43" s="21"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" ns3:dyDescent="0.3">
       <c r="A44" s="20" t="s">
         <v>69</v>
       </c>
@@ -16254,7 +16266,7 @@
       </c>
       <c r="G44" s="21"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" ns3:dyDescent="0.3">
       <c r="A45" s="20" t="s">
         <v>72</v>
       </c>
@@ -16273,7 +16285,7 @@
       </c>
       <c r="G45" s="21"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" ns3:dyDescent="0.3">
       <c r="A46" s="20" t="s">
         <v>75</v>
       </c>
@@ -16292,7 +16304,7 @@
       </c>
       <c r="G46" s="21"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" ns3:dyDescent="0.3">
       <c r="A47" s="20" t="s">
         <v>78</v>
       </c>
@@ -16311,7 +16323,7 @@
       </c>
       <c r="G47" s="21"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" ns3:dyDescent="0.3">
       <c r="A48" s="20" t="s">
         <v>87</v>
       </c>
@@ -16330,7 +16342,7 @@
       </c>
       <c r="G48" s="21"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" ns3:dyDescent="0.3">
       <c r="A49" s="20" t="s">
         <v>90</v>
       </c>
@@ -16349,7 +16361,7 @@
       </c>
       <c r="G49" s="21"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" ns3:dyDescent="0.3">
       <c r="A50" s="20" t="s">
         <v>93</v>
       </c>
@@ -16368,7 +16380,7 @@
       </c>
       <c r="G50" s="21"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" ns3:dyDescent="0.3">
       <c r="A51" s="20" t="s">
         <v>96</v>
       </c>
@@ -16387,7 +16399,7 @@
       </c>
       <c r="G51" s="21"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" ns3:dyDescent="0.3">
       <c r="A52" s="20" t="s">
         <v>170</v>
       </c>
@@ -16406,7 +16418,7 @@
       </c>
       <c r="G52" s="21"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" ns3:dyDescent="0.3">
       <c r="A53" s="20" t="s">
         <v>173</v>
       </c>
@@ -16425,7 +16437,7 @@
       </c>
       <c r="G53" s="21"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" ns3:dyDescent="0.3">
       <c r="A54" s="20" t="s">
         <v>257</v>
       </c>
@@ -16444,7 +16456,7 @@
       </c>
       <c r="G54" s="21"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" ns3:dyDescent="0.3">
       <c r="A55" s="20" t="s">
         <v>280</v>
       </c>
@@ -16463,7 +16475,7 @@
       </c>
       <c r="G55" s="21"/>
     </row>
-    <row r="56" spans="1:7" s="7" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" s="7" customFormat="1" ht="31.2" ns3:dyDescent="0.3">
       <c r="A56" s="20" t="s">
         <v>129</v>
       </c>
@@ -16481,6 +16493,25 @@
         <v>897</v>
       </c>
       <c r="G56" s="21"/>
+    </row>
+    <row r="57" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
+      <c r="A57" s="16" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B57" s="16" t="s">
+        <v>905</v>
+      </c>
+      <c r="C57" s="16" t="s">
+        <v>1322</v>
+      </c>
+      <c r="D57" s="17" t="s">
+        <v>1323</v>
+      </c>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17" t="s">
+        <v>897</v>
+      </c>
+      <c r="G57" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
Apply SP 800-73-5 CHUID field rules in existing PIV cases
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1339">
   <si>
     <t>Document</t>
   </si>
@@ -4007,6 +4007,51 @@
   </si>
   <si>
     <t>Reject eliminated CCC tags E3 and B4 under SP 800-73-5 Part 1 Appendix A Table 9.</t>
+  </si>
+  <si>
+    <t>CHUID tag 0x30 is first</t>
+  </si>
+  <si>
+    <t>73-5.43</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_43</t>
+  </si>
+  <si>
+    <t>CHUID tags 0x32 and 0x33 are absent</t>
+  </si>
+  <si>
+    <t>73-5.11</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_11</t>
+  </si>
+  <si>
+    <t>CHUID tag 0x34 immediately follows tag 0x30</t>
+  </si>
+  <si>
+    <t>73-5.45</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_45</t>
+  </si>
+  <si>
+    <t>CHUID tag 0xEE is absent</t>
+  </si>
+  <si>
+    <t>73-5.9</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_9</t>
+  </si>
+  <si>
+    <t>No CHUID tags other than (0x30, 0x34, 0x35, 0x36, 0x3E, 0xFE) are present</t>
+  </si>
+  <si>
+    <t>73-5.17</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_17</t>
   </si>
 </sst>
 </file>
@@ -5250,10 +5295,10 @@
         <v>61</v>
       </c>
       <c r="C24" s="54" t="s">
-        <v>62</v>
+        <v>1324</v>
       </c>
       <c r="D24" s="54" t="s">
-        <v>63</v>
+        <v>1325</v>
       </c>
       <c r="E24" s="54"/>
       <c r="F24" s="54" t="s">
@@ -5268,10 +5313,10 @@
         <v>64</v>
       </c>
       <c r="C25" s="45" t="s">
-        <v>65</v>
+        <v>1327</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>66</v>
+        <v>1328</v>
       </c>
       <c r="E25" s="45"/>
       <c r="F25" s="45" t="s">
@@ -5304,10 +5349,10 @@
         <v>70</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>71</v>
+        <v>1330</v>
       </c>
       <c r="D27" s="54" t="s">
-        <v>72</v>
+        <v>1331</v>
       </c>
       <c r="E27" s="54"/>
       <c r="F27" s="54" t="s">
@@ -5466,10 +5511,10 @@
         <v>97</v>
       </c>
       <c r="C36" s="45" t="s">
-        <v>98</v>
+        <v>1333</v>
       </c>
       <c r="D36" s="45" t="s">
-        <v>99</v>
+        <v>1334</v>
       </c>
       <c r="E36" s="45"/>
       <c r="F36" s="45" t="s">
@@ -5484,10 +5529,10 @@
         <v>100</v>
       </c>
       <c r="C37" s="45" t="s">
-        <v>101</v>
+        <v>1336</v>
       </c>
       <c r="D37" s="45" t="s">
-        <v>102</v>
+        <v>1337</v>
       </c>
       <c r="E37" s="45"/>
       <c r="F37" s="45" t="s">
@@ -15601,16 +15646,16 @@
     </row>
     <row r="10" spans="1:7" ns3:dyDescent="0.3">
       <c r="A10" s="16" t="s">
-        <v>99</v>
+        <v>1334</v>
       </c>
       <c r="B10" s="16" t="s">
         <v>916</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>918</v>
+        <v>1335</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>98</v>
+        <v>1333</v>
       </c>
       <c r="E10" s="17"/>
       <c r="F10" s="17" t="s">
@@ -15639,16 +15684,16 @@
     </row>
     <row r="12" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>66</v>
+        <v>1328</v>
       </c>
       <c r="B12" s="16" t="s">
         <v>916</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>921</v>
+        <v>1329</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>65</v>
+        <v>1327</v>
       </c>
       <c r="E12" s="17"/>
       <c r="F12" s="17" t="s">
@@ -15755,16 +15800,16 @@
     </row>
     <row r="18" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A18" s="16" t="s">
-        <v>102</v>
+        <v>1337</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>916</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>930</v>
+        <v>1338</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>101</v>
+        <v>1336</v>
       </c>
       <c r="E18" s="17"/>
       <c r="F18" s="17" t="s">
@@ -16230,16 +16275,16 @@
     </row>
     <row r="43" spans="1:7" ns3:dyDescent="0.3">
       <c r="A43" s="20" t="s">
-        <v>63</v>
+        <v>1325</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>916</v>
       </c>
       <c r="C43" s="20" t="s">
-        <v>969</v>
+        <v>1326</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>970</v>
+        <v>1324</v>
       </c>
       <c r="E43" s="21"/>
       <c r="F43" s="17" t="s">
@@ -16268,16 +16313,16 @@
     </row>
     <row r="45" spans="1:7" ns3:dyDescent="0.3">
       <c r="A45" s="20" t="s">
-        <v>72</v>
+        <v>1331</v>
       </c>
       <c r="B45" s="20" t="s">
         <v>916</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>973</v>
+        <v>1332</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>974</v>
+        <v>1330</v>
       </c>
       <c r="E45" s="21"/>
       <c r="F45" s="17" t="s">

</xml_diff>

<commit_message>
Validate current PIV CHUID Cardholder UUIDs
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1344">
   <si>
     <t>Document</t>
   </si>
@@ -4052,6 +4052,21 @@
   </si>
   <si>
     <t>sp800_73_5_Test_17</t>
+  </si>
+  <si>
+    <t>Optional CHUID tag 0x36 follows tag 0x35 and contains a version 4 Cardholder UUID</t>
+  </si>
+  <si>
+    <t>73-5.13</t>
+  </si>
+  <si>
+    <t>Optional CHUID Cardholder UUID is a 16-byte RFC 4122 version 4 value</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_13</t>
+  </si>
+  <si>
+    <t>Optional CHUID Cardholder UUID follows tag 0x35 and is RFC 4122 version 4</t>
   </si>
 </sst>
 </file>
@@ -5403,10 +5418,10 @@
         <v>79</v>
       </c>
       <c r="C30" s="45" t="s">
-        <v>80</v>
+        <v>1339</v>
       </c>
       <c r="D30" s="45" t="s">
-        <v>81</v>
+        <v>1340</v>
       </c>
       <c r="E30" s="45"/>
       <c r="F30" s="45" t="s">
@@ -5601,10 +5616,10 @@
         <v>112</v>
       </c>
       <c r="C41" s="45" t="s">
-        <v>113</v>
+        <v>1341</v>
       </c>
       <c r="D41" s="45" t="s">
-        <v>81</v>
+        <v>1340</v>
       </c>
       <c r="E41" s="45"/>
       <c r="F41" s="45" t="s">
@@ -15722,16 +15737,16 @@
     </row>
     <row r="14" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
       <c r="A14" s="16" t="s">
-        <v>81</v>
+        <v>1340</v>
       </c>
       <c r="B14" s="16" t="s">
         <v>916</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>923</v>
+        <v>1342</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>924</v>
+        <v>1343</v>
       </c>
       <c r="E14" s="17"/>
       <c r="F14" s="17" t="s">

</xml_diff>

<commit_message>
Remove MSCUID from current PIV active certificate checks
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1353">
   <si>
     <t>Document</t>
   </si>
@@ -4067,6 +4067,33 @@
   </si>
   <si>
     <t>Optional CHUID Cardholder UUID follows tag 0x35 and is RFC 4122 version 4</t>
+  </si>
+  <si>
+    <t>Active certificate container excludes MSCUID tag 0x72 (SP 800-73-5 Tables 11, 16-18)</t>
+  </si>
+  <si>
+    <t>73-5.20</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_20</t>
+  </si>
+  <si>
+    <t>Tag 0xFE immediately follows tag 0x71 in an active certificate container (SP 800-73-5 Tables 11, 16-18)</t>
+  </si>
+  <si>
+    <t>73-5.21</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_21</t>
+  </si>
+  <si>
+    <t>Only tags 0x70, 0x71 and 0xFE occur in an active certificate container (SP 800-73-5 Tables 11, 16-18)</t>
+  </si>
+  <si>
+    <t>73-5.22</t>
+  </si>
+  <si>
+    <t>sp800_73_5_Test_22</t>
   </si>
 </sst>
 </file>
@@ -5806,10 +5833,10 @@
         <v>133</v>
       </c>
       <c r="C52" s="45" t="s">
-        <v>134</v>
+        <v>1344</v>
       </c>
       <c r="D52" s="45" t="s">
-        <v>135</v>
+        <v>1345</v>
       </c>
       <c r="E52" s="45"/>
       <c r="F52" s="45" t="s">
@@ -5824,10 +5851,10 @@
         <v>136</v>
       </c>
       <c r="C53" s="45" t="s">
-        <v>137</v>
+        <v>1347</v>
       </c>
       <c r="D53" s="45" t="s">
-        <v>138</v>
+        <v>1348</v>
       </c>
       <c r="E53" s="45"/>
       <c r="F53" s="45" t="s">
@@ -5842,10 +5869,10 @@
         <v>139</v>
       </c>
       <c r="C54" s="45" t="s">
-        <v>140</v>
+        <v>1350</v>
       </c>
       <c r="D54" s="45" t="s">
-        <v>141</v>
+        <v>1351</v>
       </c>
       <c r="E54" s="45"/>
       <c r="F54" s="45" t="s">
@@ -6566,10 +6593,10 @@
         <v>209</v>
       </c>
       <c r="C96" s="45" t="s">
-        <v>134</v>
+        <v>1344</v>
       </c>
       <c r="D96" s="45" t="s">
-        <v>135</v>
+        <v>1345</v>
       </c>
       <c r="E96" s="45"/>
       <c r="F96" s="45" t="s">
@@ -6584,10 +6611,10 @@
         <v>210</v>
       </c>
       <c r="C97" s="45" t="s">
-        <v>140</v>
+        <v>1350</v>
       </c>
       <c r="D97" s="45" t="s">
-        <v>141</v>
+        <v>1351</v>
       </c>
       <c r="E97" s="45"/>
       <c r="F97" s="45" t="s">
@@ -6602,10 +6629,10 @@
         <v>211</v>
       </c>
       <c r="C98" s="45" t="s">
-        <v>137</v>
+        <v>1347</v>
       </c>
       <c r="D98" s="45" t="s">
-        <v>138</v>
+        <v>1348</v>
       </c>
       <c r="E98" s="45"/>
       <c r="F98" s="45" t="s">
@@ -6774,10 +6801,10 @@
         <v>223</v>
       </c>
       <c r="C108" s="45" t="s">
-        <v>134</v>
+        <v>1344</v>
       </c>
       <c r="D108" s="45" t="s">
-        <v>135</v>
+        <v>1345</v>
       </c>
       <c r="E108" s="45"/>
       <c r="F108" s="45" t="s">
@@ -6792,10 +6819,10 @@
         <v>224</v>
       </c>
       <c r="C109" s="45" t="s">
-        <v>137</v>
+        <v>1347</v>
       </c>
       <c r="D109" s="45" t="s">
-        <v>138</v>
+        <v>1348</v>
       </c>
       <c r="E109" s="45"/>
       <c r="F109" s="45" t="s">
@@ -6810,10 +6837,10 @@
         <v>225</v>
       </c>
       <c r="C110" s="45" t="s">
-        <v>140</v>
+        <v>1350</v>
       </c>
       <c r="D110" s="45" t="s">
-        <v>141</v>
+        <v>1351</v>
       </c>
       <c r="E110" s="45"/>
       <c r="F110" s="45" t="s">
@@ -6982,10 +7009,10 @@
         <v>237</v>
       </c>
       <c r="C120" s="45" t="s">
-        <v>134</v>
+        <v>1344</v>
       </c>
       <c r="D120" s="45" t="s">
-        <v>135</v>
+        <v>1345</v>
       </c>
       <c r="E120" s="45"/>
       <c r="F120" s="45" t="s">
@@ -7000,10 +7027,10 @@
         <v>238</v>
       </c>
       <c r="C121" s="45" t="s">
-        <v>137</v>
+        <v>1347</v>
       </c>
       <c r="D121" s="45" t="s">
-        <v>138</v>
+        <v>1348</v>
       </c>
       <c r="E121" s="45"/>
       <c r="F121" s="45" t="s">
@@ -7018,10 +7045,10 @@
         <v>239</v>
       </c>
       <c r="C122" s="45" t="s">
-        <v>140</v>
+        <v>1350</v>
       </c>
       <c r="D122" s="45" t="s">
-        <v>141</v>
+        <v>1351</v>
       </c>
       <c r="E122" s="45"/>
       <c r="F122" s="45" t="s">
@@ -15872,16 +15899,16 @@
     </row>
     <row r="21" spans="1:7" ns3:dyDescent="0.3">
       <c r="A21" s="16" t="s">
-        <v>135</v>
+        <v>1345</v>
       </c>
       <c r="B21" s="16" t="s">
         <v>932</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>936</v>
+        <v>1346</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>134</v>
+        <v>1344</v>
       </c>
       <c r="E21" s="17"/>
       <c r="F21" s="17" t="s">
@@ -15891,16 +15918,16 @@
     </row>
     <row r="22" spans="1:7" ns3:dyDescent="0.3">
       <c r="A22" s="16" t="s">
-        <v>138</v>
+        <v>1348</v>
       </c>
       <c r="B22" s="16" t="s">
         <v>932</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>937</v>
+        <v>1349</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>137</v>
+        <v>1347</v>
       </c>
       <c r="E22" s="17"/>
       <c r="F22" s="17" t="s">
@@ -15910,16 +15937,16 @@
     </row>
     <row r="23" spans="1:7" ns3:dyDescent="0.3">
       <c r="A23" s="16" t="s">
-        <v>141</v>
+        <v>1351</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>932</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>938</v>
+        <v>1352</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>140</v>
+        <v>1350</v>
       </c>
       <c r="E23" s="17"/>
       <c r="F23" s="17" t="s">

</xml_diff>

<commit_message>
Validate optional PIV Authentication Cardholder UUID SAN
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1356">
   <si>
     <t>Document</t>
   </si>
@@ -4094,6 +4094,15 @@
   </si>
   <si>
     <t>sp800_73_5_Test_22</t>
+  </si>
+  <si>
+    <t>PIV Authentication certificate SAN contains the CHUID Card UUID and, if present, a version 4 Cardholder UUID matching CHUID tag 0x36 (SP 800-73-5 Sections 3.4.1-3.4.2)</t>
+  </si>
+  <si>
+    <t>PKIX.27.current</t>
+  </si>
+  <si>
+    <t>PKIX_Test_27_current</t>
   </si>
 </sst>
 </file>
@@ -12319,10 +12328,10 @@
         <v>708</v>
       </c>
       <c r="C370" s="52" t="s">
-        <v>709</v>
+        <v>1353</v>
       </c>
       <c r="D370" s="45" t="s">
-        <v>710</v>
+        <v>1354</v>
       </c>
       <c r="E370" s="52"/>
       <c r="F370" s="45" t="s">
@@ -14719,7 +14728,7 @@
         <v>709</v>
       </c>
       <c r="D452" s="45" t="s">
-        <v>710</v>
+        <v>1354</v>
       </c>
       <c r="E452" s="52"/>
       <c r="F452" s="45" t="s">
@@ -20385,16 +20394,16 @@
     </row>
     <row r="28" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A28" s="63" t="s">
-        <v>710</v>
+        <v>1354</v>
       </c>
       <c r="B28" s="63" t="s">
         <v>1191</v>
       </c>
       <c r="C28" s="63" t="s">
-        <v>1249</v>
+        <v>1355</v>
       </c>
       <c r="D28" s="63" t="s">
-        <v>709</v>
+        <v>1353</v>
       </c>
       <c r="E28" s="66" t="s">
         <v>1250</v>

</xml_diff>

<commit_message>
Check current PIV signature algorithms in existing cases
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="1361">
   <si>
     <t>Document</t>
   </si>
@@ -4103,6 +4103,21 @@
   </si>
   <si>
     <t>PKIX_Test_27_current</t>
+  </si>
+  <si>
+    <t>Certificate signature algorithm and parameters use SP 800-78-5 Section 3.2.1 Tables 2-3: RSA SHA-256/384 with PKCS #1 v1.5 or PSS, or ECDSA SHA-256/384</t>
+  </si>
+  <si>
+    <t>78.3.current</t>
+  </si>
+  <si>
+    <t>CHUID CMS SignerInfo algorithm and digest use SP 800-78-5 Section 3.2.1 Tables 2-3 and the signature verifies</t>
+  </si>
+  <si>
+    <t>sp800_78_Test_3_current</t>
+  </si>
+  <si>
+    <t>PIV certificate or CHUID CMS signature algorithm, digest and parameters satisfy SP 800-78-5 Section 3.2.1 Tables 2-3</t>
   </si>
 </sst>
 </file>
@@ -12005,10 +12020,10 @@
         <v>669</v>
       </c>
       <c r="C351" s="52" t="s">
-        <v>670</v>
-      </c>
-      <c r="D351" s="45">
-        <v>78.3</v>
+        <v>1356</v>
+      </c>
+      <c r="D351" s="45" t="s">
+        <v>1357</v>
       </c>
       <c r="E351" s="45"/>
       <c r="F351" s="45" t="s">
@@ -13580,10 +13595,10 @@
         <v>738</v>
       </c>
       <c r="C384" s="52" t="s">
-        <v>670</v>
+        <v>1356</v>
       </c>
       <c r="D384" s="45" t="s">
-        <v>739</v>
+        <v>1357</v>
       </c>
       <c r="E384" s="52"/>
       <c r="F384" s="45" t="s">
@@ -13966,10 +13981,10 @@
         <v>773</v>
       </c>
       <c r="C407" s="52" t="s">
-        <v>670</v>
-      </c>
-      <c r="D407" s="45">
-        <v>78.3</v>
+        <v>1356</v>
+      </c>
+      <c r="D407" s="45" t="s">
+        <v>1357</v>
       </c>
       <c r="E407" s="52"/>
       <c r="F407" s="45" t="s">
@@ -14352,10 +14367,10 @@
         <v>803</v>
       </c>
       <c r="C430" s="52" t="s">
-        <v>670</v>
-      </c>
-      <c r="D430" s="45">
-        <v>78.3</v>
+        <v>1356</v>
+      </c>
+      <c r="D430" s="45" t="s">
+        <v>1357</v>
       </c>
       <c r="E430" s="52"/>
       <c r="F430" s="45" t="s">
@@ -14986,10 +15001,10 @@
         <v>860</v>
       </c>
       <c r="C469" s="52" t="s">
-        <v>670</v>
-      </c>
-      <c r="D469" s="45">
-        <v>78.3</v>
+        <v>1358</v>
+      </c>
+      <c r="D469" s="45" t="s">
+        <v>1357</v>
       </c>
       <c r="E469" s="52"/>
       <c r="F469" s="45" t="s">
@@ -19291,16 +19306,16 @@
     </row>
     <row r="4" spans="1:256" ht="78" ns3:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>739</v>
+        <v>1357</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>1183</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1189</v>
+        <v>1359</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>670</v>
+        <v>1360</v>
       </c>
       <c r="E4" s="23"/>
       <c r="F4" s="11" t="s">

</xml_diff>

<commit_message>
Route PIV facial image checks to existing biometric atoms
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -9302,7 +9302,7 @@
         <v>491</v>
       </c>
       <c r="D252" s="45" t="s">
-        <v>283</v>
+        <v>1070</v>
       </c>
       <c r="E252" s="45"/>
       <c r="F252" s="45" t="s">
@@ -9320,7 +9320,7 @@
         <v>493</v>
       </c>
       <c r="D253" s="45" t="s">
-        <v>283</v>
+        <v>1073</v>
       </c>
       <c r="E253" s="45"/>
       <c r="F253" s="45" t="s">
@@ -9338,7 +9338,7 @@
         <v>495</v>
       </c>
       <c r="D254" s="45" t="s">
-        <v>283</v>
+        <v>1076</v>
       </c>
       <c r="E254" s="45"/>
       <c r="F254" s="45" t="s">
@@ -9356,7 +9356,7 @@
         <v>497</v>
       </c>
       <c r="D255" s="45" t="s">
-        <v>283</v>
+        <v>1079</v>
       </c>
       <c r="E255" s="45"/>
       <c r="F255" s="45" t="s">

</xml_diff>

<commit_message>
Check PIV Key History fields through existing case
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -7569,8 +7569,10 @@
       <c r="C151" s="45" t="s">
         <v>299</v>
       </c>
-      <c r="D151" s="45" t="s">
-        <v>283</v>
+      <c r="D151" s="45" t="inlineStr">
+        <is>
+          <t>73-4.57</t>
+        </is>
       </c>
       <c r="E151" s="45"/>
       <c r="F151" s="45" t="s">
@@ -15522,7 +15524,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMK57"/>
+  <dimension ref="A1:AMK58"/>
   <sheetFormatPr defaultRowHeight="15.6" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5" style="13" customWidth="1"/>
@@ -16623,6 +16625,35 @@
         <v>897</v>
       </c>
       <c r="G57" s="17"/>
+    </row>
+    <row r="58" spans="1:7" ht="31.2" ns3:dyDescent="0.3">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>73-4.57</t>
+        </is>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>gov.gsa.pivconformance.conformancelib.tests.SP800_73_4KeyHistoryTests</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>sp800_73_4_Test_57</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Verify Key History counts, conditional URL, field lengths and tag order under SP 800-73-5 Part 1 Table 20.</t>
+        </is>
+      </c>
+      <c r="E58" s="17"/>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G58" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
Repair audited PIV assertions and preserve intended failure paths
</commit_message>
<xml_diff>
--- a/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
+++ b/conformancelib/testdata/PIV_ICAM_Test_Cards.xlsx
@@ -18852,8 +18852,10 @@
       <c r="B23" s="15" t="s">
         <v>1115</v>
       </c>
-      <c r="C23" s="15" t="s">
-        <v>1162</v>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CMS_Test_23_current</t>
+        </is>
       </c>
       <c r="D23" s="15" t="s">
         <v>569</v>

</xml_diff>